<commit_message>
docs: qa-roadmap updated TC-12 test
</commit_message>
<xml_diff>
--- a/docs/QA_Roadmap_Natalia.xlsx
+++ b/docs/QA_Roadmap_Natalia.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="118">
   <si>
     <t>ID</t>
   </si>
@@ -294,9 +294,6 @@
   </si>
   <si>
     <t>Ordenamiento de nombre de los productos (A to Z)</t>
-  </si>
-  <si>
-    <t>Pendiente</t>
   </si>
   <si>
     <r>
@@ -372,28 +369,88 @@
     </r>
   </si>
   <si>
+    <t>Verificar estado inicial del carrito.</t>
+  </si>
+  <si>
+    <t>El badge (.shopping_cart_badge) no es visible o es 0.</t>
+  </si>
+  <si>
+    <t>Click en "Add to Cart" de un producto específico.</t>
+  </si>
+  <si>
+    <t>El botón cambia a "Remove".</t>
+  </si>
+  <si>
+    <t>Validar que el badge muestra el número "1".</t>
+  </si>
+  <si>
+    <t>El contador se incrementa correctamente.</t>
+  </si>
+  <si>
+    <t>TC-12</t>
+  </si>
+  <si>
+    <t>Validar la persistencia de productos en el carrito</t>
+  </si>
+  <si>
+    <t>.shopping_cart_link, .inventory_item_name</t>
+  </si>
+  <si>
+    <t>Add a product to the cart.</t>
+  </si>
+  <si>
+    <t>The badge shows "1".</t>
+  </si>
+  <si>
+    <t>Click the Cart Icon (Navigation).</t>
+  </si>
+  <si>
+    <t>The browser navigates to /cart.html.</t>
+  </si>
+  <si>
+    <t>Verify the product name in the cart.</t>
+  </si>
+  <si>
+    <t>The name matches the added product.</t>
+  </si>
+  <si>
+    <t>TC-13</t>
+  </si>
+  <si>
+    <t>Verificar la eliminación del producto del carrito</t>
+  </si>
+  <si>
+    <t>Pendiente</t>
+  </si>
+  <si>
+    <t>.cart_button, .removed_cart_item</t>
+  </si>
+  <si>
     <t>❌ NO</t>
   </si>
   <si>
     <t>PENDIENTE 🟡</t>
   </si>
   <si>
-    <t>Verificar estado inicial del carrito.</t>
-  </si>
-  <si>
-    <t>El badge (.shopping_cart_badge) no es visible o es 0.</t>
-  </si>
-  <si>
-    <t>Click en "Add to Cart" de un producto específico.</t>
-  </si>
-  <si>
-    <t>El botón cambia a "Remove".</t>
-  </si>
-  <si>
-    <t>Validar que el badge muestra el número "1".</t>
-  </si>
-  <si>
-    <t>El contador se incrementa correctamente.</t>
+    <t>Pending</t>
+  </si>
+  <si>
+    <t>Add an item and navigate to the cart.</t>
+  </si>
+  <si>
+    <t>The item is visible in the cart.</t>
+  </si>
+  <si>
+    <t>Click the "Remove" button in the cart.</t>
+  </si>
+  <si>
+    <t>The item is removed from the list.</t>
+  </si>
+  <si>
+    <t>Verify the badge count updates.</t>
+  </si>
+  <si>
+    <t>The badge decreases or disappears.</t>
   </si>
   <si>
     <t>PENDIENTE 🟡,</t>
@@ -474,7 +531,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="52">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -514,6 +571,9 @@
     <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="top"/>
+    </xf>
     <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
@@ -529,9 +589,6 @@
     <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="top"/>
-    </xf>
     <xf borderId="0" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="0"/>
     </xf>
@@ -564,6 +621,54 @@
     </xf>
     <xf borderId="0" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
@@ -899,7 +1004,7 @@
     <col customWidth="1" min="7" max="7" width="13.13"/>
     <col customWidth="1" min="8" max="8" width="15.63"/>
     <col customWidth="1" min="9" max="9" width="4.75"/>
-    <col customWidth="1" min="10" max="10" width="63.75"/>
+    <col customWidth="1" min="10" max="10" width="38.25"/>
     <col customWidth="1" min="11" max="11" width="56.13"/>
     <col customWidth="1" min="12" max="12" width="8.5"/>
     <col customWidth="1" min="13" max="27" width="20.75"/>
@@ -2160,10 +2265,10 @@
         <v>65</v>
       </c>
       <c r="D35" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E35" s="4" t="s">
         <v>75</v>
-      </c>
-      <c r="E35" s="4" t="s">
-        <v>76</v>
       </c>
       <c r="F35" s="1" t="s">
         <v>16</v>
@@ -2279,10 +2384,10 @@
         <v>4.0</v>
       </c>
       <c r="J38" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="K38" s="9" t="s">
         <v>77</v>
-      </c>
-      <c r="K38" s="9" t="s">
-        <v>78</v>
       </c>
       <c r="L38" s="1" t="s">
         <v>20</v>
@@ -2300,19 +2405,19 @@
     </row>
     <row r="41">
       <c r="A41" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="B41" s="1" t="s">
         <v>79</v>
-      </c>
-      <c r="B41" s="1" t="s">
-        <v>80</v>
       </c>
       <c r="C41" s="9" t="s">
         <v>65</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>75</v>
+        <v>14</v>
       </c>
       <c r="E41" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F41" s="1" t="s">
         <v>16</v>
@@ -2369,10 +2474,10 @@
         <v>4.0</v>
       </c>
       <c r="J44" s="9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="K44" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="L44" s="1" t="s">
         <v>20</v>
@@ -2380,40 +2485,40 @@
     </row>
     <row r="45">
       <c r="A45" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="B45" s="12" t="s">
         <v>83</v>
-      </c>
-      <c r="B45" s="12" t="s">
-        <v>84</v>
       </c>
       <c r="C45" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="D45" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E45" s="13" t="s">
-        <v>85</v>
-      </c>
-      <c r="F45" s="12" t="s">
-        <v>86</v>
-      </c>
-      <c r="G45" s="12" t="s">
-        <v>87</v>
-      </c>
-      <c r="H45" s="14">
+      <c r="D45" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="E45" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="F45" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="G45" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H45" s="15">
         <v>46066.0</v>
       </c>
-      <c r="I45" s="15">
+      <c r="I45" s="16">
         <v>1.0</v>
       </c>
-      <c r="J45" s="16" t="s">
+      <c r="J45" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="K45" s="17" t="s">
+      <c r="K45" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="L45" s="18" t="s">
-        <v>75</v>
+      <c r="L45" s="13" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="46">
@@ -2434,7 +2539,7 @@
         <v>22</v>
       </c>
       <c r="L46" s="22" t="s">
-        <v>75</v>
+        <v>20</v>
       </c>
     </row>
     <row r="47">
@@ -2445,17 +2550,17 @@
       <c r="F47" s="12"/>
       <c r="G47" s="12"/>
       <c r="H47" s="12"/>
-      <c r="I47" s="15">
+      <c r="I47" s="16">
         <v>3.0</v>
       </c>
-      <c r="J47" s="18" t="s">
+      <c r="J47" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="K47" s="18" t="s">
+      <c r="K47" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="L47" s="18" t="s">
-        <v>75</v>
+      <c r="L47" s="13" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="48">
@@ -2470,13 +2575,13 @@
         <v>4.0</v>
       </c>
       <c r="J48" s="20" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="K48" s="20" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="L48" s="22" t="s">
-        <v>75</v>
+        <v>20</v>
       </c>
     </row>
     <row r="49">
@@ -2491,13 +2596,13 @@
         <v>5.0</v>
       </c>
       <c r="J49" s="12" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="K49" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="L49" s="18" t="s">
-        <v>75</v>
+        <v>88</v>
+      </c>
+      <c r="L49" s="13" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="50">
@@ -2512,17 +2617,17 @@
         <v>6.0</v>
       </c>
       <c r="J50" s="20" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="K50" s="20" t="s">
-        <v>93</v>
-      </c>
-      <c r="L50" s="20" t="s">
-        <v>75</v>
+        <v>90</v>
+      </c>
+      <c r="L50" s="22" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="24"/>
+      <c r="A51" s="30"/>
       <c r="B51" s="25"/>
       <c r="C51" s="25"/>
       <c r="D51" s="25"/>
@@ -2536,25 +2641,380 @@
       <c r="L51" s="12"/>
     </row>
     <row r="52">
-      <c r="A52" s="27"/>
-      <c r="B52" s="28"/>
-      <c r="C52" s="28"/>
-      <c r="D52" s="28"/>
-      <c r="E52" s="28"/>
-      <c r="F52" s="28"/>
-      <c r="G52" s="28"/>
-      <c r="H52" s="28"/>
-      <c r="I52" s="27"/>
-      <c r="J52" s="20"/>
-      <c r="K52" s="20"/>
-      <c r="L52" s="20"/>
+      <c r="A52" s="31" t="s">
+        <v>91</v>
+      </c>
+      <c r="B52" s="32" t="s">
+        <v>92</v>
+      </c>
+      <c r="C52" s="32" t="s">
+        <v>13</v>
+      </c>
+      <c r="D52" s="22" t="s">
+        <v>14</v>
+      </c>
+      <c r="E52" s="33" t="s">
+        <v>93</v>
+      </c>
+      <c r="F52" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="G52" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H52" s="34">
+        <v>46067.0</v>
+      </c>
+      <c r="I52" s="29">
+        <v>1.0</v>
+      </c>
+      <c r="J52" s="23" t="s">
+        <v>18</v>
+      </c>
+      <c r="K52" s="35" t="s">
+        <v>19</v>
+      </c>
+      <c r="L52" s="22" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="30"/>
+      <c r="B53" s="25"/>
+      <c r="C53" s="36"/>
+      <c r="D53" s="36"/>
+      <c r="F53" s="36"/>
+      <c r="G53" s="36"/>
+      <c r="H53" s="37"/>
+      <c r="I53" s="26">
+        <v>2.0</v>
+      </c>
+      <c r="J53" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="K53" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="L53" s="13" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="31"/>
+      <c r="B54" s="28"/>
+      <c r="C54" s="32"/>
+      <c r="D54" s="32"/>
+      <c r="F54" s="32"/>
+      <c r="G54" s="32"/>
+      <c r="H54" s="34"/>
+      <c r="I54" s="29">
+        <v>3.0</v>
+      </c>
+      <c r="J54" s="22" t="s">
+        <v>54</v>
+      </c>
+      <c r="K54" s="22" t="s">
+        <v>55</v>
+      </c>
+      <c r="L54" s="22" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="38"/>
+      <c r="B55" s="38"/>
+      <c r="C55" s="38"/>
+      <c r="D55" s="38"/>
+      <c r="E55" s="18"/>
+      <c r="F55" s="38"/>
+      <c r="G55" s="38"/>
+      <c r="H55" s="39"/>
+      <c r="I55" s="40">
+        <v>4.0</v>
+      </c>
+      <c r="J55" s="38" t="s">
+        <v>94</v>
+      </c>
+      <c r="K55" s="38" t="s">
+        <v>95</v>
+      </c>
+      <c r="L55" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="M55" s="41"/>
+      <c r="N55" s="41"/>
+      <c r="O55" s="41"/>
+      <c r="P55" s="41"/>
+      <c r="Q55" s="41"/>
+      <c r="R55" s="41"/>
+      <c r="S55" s="41"/>
+      <c r="T55" s="41"/>
+      <c r="U55" s="41"/>
+      <c r="V55" s="41"/>
+      <c r="W55" s="41"/>
+      <c r="X55" s="41"/>
+      <c r="Y55" s="41"/>
+      <c r="Z55" s="41"/>
+      <c r="AA55" s="41"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="42"/>
+      <c r="B56" s="42"/>
+      <c r="C56" s="42"/>
+      <c r="D56" s="42"/>
+      <c r="E56" s="35"/>
+      <c r="F56" s="42"/>
+      <c r="G56" s="42"/>
+      <c r="H56" s="43"/>
+      <c r="I56" s="44">
+        <v>5.0</v>
+      </c>
+      <c r="J56" s="42" t="s">
+        <v>96</v>
+      </c>
+      <c r="K56" s="42" t="s">
+        <v>97</v>
+      </c>
+      <c r="L56" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="M56" s="41"/>
+      <c r="N56" s="41"/>
+      <c r="O56" s="41"/>
+      <c r="P56" s="41"/>
+      <c r="Q56" s="41"/>
+      <c r="R56" s="41"/>
+      <c r="S56" s="41"/>
+      <c r="T56" s="41"/>
+      <c r="U56" s="41"/>
+      <c r="V56" s="41"/>
+      <c r="W56" s="41"/>
+      <c r="X56" s="41"/>
+      <c r="Y56" s="41"/>
+      <c r="Z56" s="41"/>
+      <c r="AA56" s="41"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="38"/>
+      <c r="B57" s="38"/>
+      <c r="C57" s="38"/>
+      <c r="D57" s="38"/>
+      <c r="E57" s="18"/>
+      <c r="F57" s="38"/>
+      <c r="G57" s="38"/>
+      <c r="H57" s="39"/>
+      <c r="I57" s="40">
+        <v>6.0</v>
+      </c>
+      <c r="J57" s="38" t="s">
+        <v>98</v>
+      </c>
+      <c r="K57" s="38" t="s">
+        <v>99</v>
+      </c>
+      <c r="L57" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="M57" s="41"/>
+      <c r="N57" s="41"/>
+      <c r="O57" s="41"/>
+      <c r="P57" s="41"/>
+      <c r="Q57" s="41"/>
+      <c r="R57" s="41"/>
+      <c r="S57" s="41"/>
+      <c r="T57" s="41"/>
+      <c r="U57" s="41"/>
+      <c r="V57" s="41"/>
+      <c r="W57" s="41"/>
+      <c r="X57" s="41"/>
+      <c r="Y57" s="41"/>
+      <c r="Z57" s="41"/>
+      <c r="AA57" s="41"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="42"/>
+      <c r="B58" s="42"/>
+      <c r="C58" s="42"/>
+      <c r="D58" s="42"/>
+      <c r="E58" s="35"/>
+      <c r="F58" s="42"/>
+      <c r="G58" s="42"/>
+      <c r="H58" s="43"/>
+      <c r="I58" s="42"/>
+      <c r="J58" s="42"/>
+      <c r="K58" s="42"/>
+      <c r="L58" s="42"/>
+      <c r="M58" s="41"/>
+      <c r="N58" s="41"/>
+      <c r="O58" s="41"/>
+      <c r="P58" s="41"/>
+      <c r="Q58" s="41"/>
+      <c r="R58" s="41"/>
+      <c r="S58" s="41"/>
+      <c r="T58" s="41"/>
+      <c r="U58" s="41"/>
+      <c r="V58" s="41"/>
+      <c r="W58" s="41"/>
+      <c r="X58" s="41"/>
+      <c r="Y58" s="41"/>
+      <c r="Z58" s="41"/>
+      <c r="AA58" s="41"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="30" t="s">
+        <v>100</v>
+      </c>
+      <c r="B59" s="36" t="s">
+        <v>101</v>
+      </c>
+      <c r="C59" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="D59" s="36" t="s">
+        <v>102</v>
+      </c>
+      <c r="E59" s="45" t="s">
+        <v>103</v>
+      </c>
+      <c r="F59" s="36" t="s">
+        <v>104</v>
+      </c>
+      <c r="G59" s="36" t="s">
+        <v>105</v>
+      </c>
+      <c r="H59" s="37">
+        <v>46069.0</v>
+      </c>
+      <c r="I59" s="26">
+        <v>1.0</v>
+      </c>
+      <c r="J59" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="K59" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="L59" s="38" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="31"/>
+      <c r="B60" s="28"/>
+      <c r="C60" s="32"/>
+      <c r="D60" s="32"/>
+      <c r="E60" s="28"/>
+      <c r="F60" s="32"/>
+      <c r="G60" s="32"/>
+      <c r="H60" s="34"/>
+      <c r="I60" s="29">
+        <v>2.0</v>
+      </c>
+      <c r="J60" s="22" t="s">
+        <v>46</v>
+      </c>
+      <c r="K60" s="23" t="s">
+        <v>22</v>
+      </c>
+      <c r="L60" s="42" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="30"/>
+      <c r="B61" s="25"/>
+      <c r="C61" s="36"/>
+      <c r="D61" s="36"/>
+      <c r="E61" s="25"/>
+      <c r="F61" s="36"/>
+      <c r="G61" s="36"/>
+      <c r="H61" s="37"/>
+      <c r="I61" s="26">
+        <v>3.0</v>
+      </c>
+      <c r="J61" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="K61" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="L61" s="38" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="27"/>
+      <c r="B62" s="28"/>
+      <c r="C62" s="28"/>
+      <c r="D62" s="28"/>
+      <c r="E62" s="28"/>
+      <c r="F62" s="28"/>
+      <c r="G62" s="28"/>
+      <c r="H62" s="28"/>
+      <c r="I62" s="29">
+        <v>4.0</v>
+      </c>
+      <c r="J62" s="42" t="s">
+        <v>107</v>
+      </c>
+      <c r="K62" s="42" t="s">
+        <v>108</v>
+      </c>
+      <c r="L62" s="42" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="24"/>
+      <c r="B63" s="25"/>
+      <c r="C63" s="25"/>
+      <c r="D63" s="25"/>
+      <c r="E63" s="25"/>
+      <c r="F63" s="25"/>
+      <c r="G63" s="25"/>
+      <c r="H63" s="25"/>
+      <c r="I63" s="26">
+        <v>5.0</v>
+      </c>
+      <c r="J63" s="38" t="s">
+        <v>109</v>
+      </c>
+      <c r="K63" s="38" t="s">
+        <v>110</v>
+      </c>
+      <c r="L63" s="38" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="27"/>
+      <c r="B64" s="28"/>
+      <c r="C64" s="28"/>
+      <c r="D64" s="28"/>
+      <c r="E64" s="28"/>
+      <c r="F64" s="28"/>
+      <c r="G64" s="28"/>
+      <c r="H64" s="28"/>
+      <c r="I64" s="29">
+        <v>6.0</v>
+      </c>
+      <c r="J64" s="42" t="s">
+        <v>111</v>
+      </c>
+      <c r="K64" s="42" t="s">
+        <v>112</v>
+      </c>
+      <c r="L64" s="42" t="s">
+        <v>106</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="12">
     <mergeCell ref="E31:E34"/>
     <mergeCell ref="E35:E39"/>
     <mergeCell ref="E41:E44"/>
     <mergeCell ref="E45:E50"/>
+    <mergeCell ref="E52:E54"/>
     <mergeCell ref="E2:E6"/>
     <mergeCell ref="E7:E10"/>
     <mergeCell ref="E11:E14"/>
@@ -2576,10 +3036,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="9" t="s">
-        <v>86</v>
+        <v>104</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>94</v>
+        <v>113</v>
       </c>
     </row>
     <row r="2">
@@ -2609,145 +3069,145 @@
   </cols>
   <sheetData>
     <row r="45" ht="22.5" customHeight="1">
-      <c r="A45" s="30" t="s">
+      <c r="A45" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="B45" s="31" t="s">
+      <c r="B45" s="47" t="s">
         <v>1</v>
       </c>
-      <c r="C45" s="31" t="s">
+      <c r="C45" s="47" t="s">
         <v>2</v>
       </c>
-      <c r="D45" s="31" t="s">
+      <c r="D45" s="47" t="s">
         <v>3</v>
       </c>
-      <c r="E45" s="31" t="s">
+      <c r="E45" s="47" t="s">
         <v>4</v>
       </c>
-      <c r="F45" s="31" t="s">
+      <c r="F45" s="47" t="s">
         <v>5</v>
       </c>
-      <c r="G45" s="31" t="s">
+      <c r="G45" s="47" t="s">
         <v>6</v>
       </c>
-      <c r="H45" s="31" t="s">
+      <c r="H45" s="47" t="s">
         <v>7</v>
       </c>
-      <c r="I45" s="30" t="s">
+      <c r="I45" s="46" t="s">
         <v>8</v>
       </c>
-      <c r="J45" s="31" t="s">
+      <c r="J45" s="47" t="s">
         <v>9</v>
       </c>
-      <c r="K45" s="31" t="s">
+      <c r="K45" s="47" t="s">
         <v>10</v>
       </c>
-      <c r="L45" s="31" t="s">
-        <v>95</v>
+      <c r="L45" s="47" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="46" ht="22.5" customHeight="1">
-      <c r="A46" s="32" t="s">
+      <c r="A46" s="48" t="s">
+        <v>82</v>
+      </c>
+      <c r="B46" s="49" t="s">
         <v>83</v>
       </c>
-      <c r="B46" s="33" t="s">
-        <v>84</v>
-      </c>
-      <c r="C46" s="33" t="s">
+      <c r="C46" s="49" t="s">
         <v>13</v>
       </c>
-      <c r="D46" s="33" t="s">
-        <v>75</v>
-      </c>
-      <c r="E46" s="33" t="s">
-        <v>96</v>
-      </c>
-      <c r="F46" s="33" t="s">
+      <c r="D46" s="49" t="s">
+        <v>102</v>
+      </c>
+      <c r="E46" s="49" t="s">
+        <v>115</v>
+      </c>
+      <c r="F46" s="49" t="s">
+        <v>104</v>
+      </c>
+      <c r="G46" s="49" t="s">
+        <v>105</v>
+      </c>
+      <c r="H46" s="50">
+        <v>46066.0</v>
+      </c>
+      <c r="I46" s="51">
+        <v>1.0</v>
+      </c>
+      <c r="J46" s="49" t="s">
+        <v>116</v>
+      </c>
+      <c r="K46" s="49" t="s">
+        <v>117</v>
+      </c>
+      <c r="L46" s="49" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="47" ht="22.5" customHeight="1">
+      <c r="A47" s="48"/>
+      <c r="B47" s="49"/>
+      <c r="C47" s="49"/>
+      <c r="D47" s="49"/>
+      <c r="E47" s="49"/>
+      <c r="F47" s="49"/>
+      <c r="G47" s="49"/>
+      <c r="H47" s="49"/>
+      <c r="I47" s="51">
+        <v>2.0</v>
+      </c>
+      <c r="J47" s="49" t="s">
+        <v>85</v>
+      </c>
+      <c r="K47" s="49" t="s">
         <v>86</v>
       </c>
-      <c r="G46" s="33" t="s">
+      <c r="L47" s="49" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="48" ht="22.5" customHeight="1">
+      <c r="A48" s="48"/>
+      <c r="B48" s="49"/>
+      <c r="C48" s="49"/>
+      <c r="D48" s="49"/>
+      <c r="E48" s="49"/>
+      <c r="F48" s="49"/>
+      <c r="G48" s="49"/>
+      <c r="H48" s="49"/>
+      <c r="I48" s="51">
+        <v>3.0</v>
+      </c>
+      <c r="J48" s="49" t="s">
         <v>87</v>
       </c>
-      <c r="H46" s="34">
-        <v>46066.0</v>
-      </c>
-      <c r="I46" s="35">
-        <v>1.0</v>
-      </c>
-      <c r="J46" s="33" t="s">
-        <v>97</v>
-      </c>
-      <c r="K46" s="33" t="s">
-        <v>98</v>
-      </c>
-      <c r="L46" s="33" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="47" ht="22.5" customHeight="1">
-      <c r="A47" s="32"/>
-      <c r="B47" s="33"/>
-      <c r="C47" s="33"/>
-      <c r="D47" s="33"/>
-      <c r="E47" s="33"/>
-      <c r="F47" s="33"/>
-      <c r="G47" s="33"/>
-      <c r="H47" s="33"/>
-      <c r="I47" s="35">
-        <v>2.0</v>
-      </c>
-      <c r="J47" s="33" t="s">
+      <c r="K48" s="49" t="s">
         <v>88</v>
       </c>
-      <c r="K47" s="33" t="s">
+      <c r="L48" s="49" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="49" ht="22.5" customHeight="1">
+      <c r="A49" s="48"/>
+      <c r="B49" s="49"/>
+      <c r="C49" s="49"/>
+      <c r="D49" s="49"/>
+      <c r="E49" s="49"/>
+      <c r="F49" s="49"/>
+      <c r="G49" s="49"/>
+      <c r="H49" s="49"/>
+      <c r="I49" s="51">
+        <v>4.0</v>
+      </c>
+      <c r="J49" s="49" t="s">
         <v>89</v>
       </c>
-      <c r="L47" s="33" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="48" ht="22.5" customHeight="1">
-      <c r="A48" s="32"/>
-      <c r="B48" s="33"/>
-      <c r="C48" s="33"/>
-      <c r="D48" s="33"/>
-      <c r="E48" s="33"/>
-      <c r="F48" s="33"/>
-      <c r="G48" s="33"/>
-      <c r="H48" s="33"/>
-      <c r="I48" s="35">
-        <v>3.0</v>
-      </c>
-      <c r="J48" s="33" t="s">
+      <c r="K49" s="49" t="s">
         <v>90</v>
       </c>
-      <c r="K48" s="33" t="s">
-        <v>91</v>
-      </c>
-      <c r="L48" s="33" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="49" ht="22.5" customHeight="1">
-      <c r="A49" s="32"/>
-      <c r="B49" s="33"/>
-      <c r="C49" s="33"/>
-      <c r="D49" s="33"/>
-      <c r="E49" s="33"/>
-      <c r="F49" s="33"/>
-      <c r="G49" s="33"/>
-      <c r="H49" s="33"/>
-      <c r="I49" s="35">
-        <v>4.0</v>
-      </c>
-      <c r="J49" s="33" t="s">
-        <v>92</v>
-      </c>
-      <c r="K49" s="33" t="s">
-        <v>93</v>
-      </c>
-      <c r="L49" s="33" t="s">
-        <v>75</v>
+      <c r="L49" s="49" t="s">
+        <v>102</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: Add TC-13 diagnostic page and codegen documentation
</commit_message>
<xml_diff>
--- a/docs/QA_Roadmap_Natalia.xlsx
+++ b/docs/QA_Roadmap_Natalia.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="119">
   <si>
     <t>ID</t>
   </si>
@@ -393,7 +393,22 @@
     <t>Validar la persistencia de productos en el carrito</t>
   </si>
   <si>
-    <t>.shopping_cart_link, .inventory_item_name</t>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <b val="0"/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">[data-test="login-button"], [data-test="username"], [data-test="password"], .inventory_list, .inventory_item, .title, .shopping_cart_badge, .btn_inventory., </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <b/>
+        <color theme="1"/>
+      </rPr>
+      <t>shopping_cart_link, .inventory_item_name</t>
+    </r>
   </si>
   <si>
     <t>Add a product to the cart.</t>
@@ -420,46 +435,64 @@
     <t>Verificar la eliminación del producto del carrito</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <b val="0"/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">[data-test="login-button"], [data-test="username"], [data-test="password"], .inventory_list, .inventory_item, .title, .shopping_cart_badge, .btn_inventory., shopping_cart_link, .inventory_item_name, </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <b/>
+        <color theme="1"/>
+      </rPr>
+      <t>.cart_item, '[data-test="continue-shopping"]'</t>
+    </r>
+  </si>
+  <si>
+    <t>✅ SÍ (Playwright) PASSED 🟢</t>
+  </si>
+  <si>
+    <t>16/02/2026 -19/02/2026</t>
+  </si>
+  <si>
+    <t>Add an item and navigate to the cart.</t>
+  </si>
+  <si>
+    <t>The item is visible in the cart.</t>
+  </si>
+  <si>
+    <t>Click the "Remove" button in the cart.</t>
+  </si>
+  <si>
+    <t>The item is removed from the list.</t>
+  </si>
+  <si>
+    <t>Verify the badge count updates.</t>
+  </si>
+  <si>
+    <t>The badge decreases or disappears.</t>
+  </si>
+  <si>
+    <t>❌ NO</t>
+  </si>
+  <si>
+    <t>PENDIENTE 🟡,</t>
+  </si>
+  <si>
+    <t>Estado 2</t>
+  </si>
+  <si>
     <t>Pendiente</t>
   </si>
   <si>
-    <t>.cart_button, .removed_cart_item</t>
-  </si>
-  <si>
-    <t>❌ NO</t>
+    <t>.shopping_cart_badge, .btn_inventory</t>
   </si>
   <si>
     <t>PENDIENTE 🟡</t>
-  </si>
-  <si>
-    <t>Pending</t>
-  </si>
-  <si>
-    <t>Add an item and navigate to the cart.</t>
-  </si>
-  <si>
-    <t>The item is visible in the cart.</t>
-  </si>
-  <si>
-    <t>Click the "Remove" button in the cart.</t>
-  </si>
-  <si>
-    <t>The item is removed from the list.</t>
-  </si>
-  <si>
-    <t>Verify the badge count updates.</t>
-  </si>
-  <si>
-    <t>The badge decreases or disappears.</t>
-  </si>
-  <si>
-    <t>PENDIENTE 🟡,</t>
-  </si>
-  <si>
-    <t>Estado 2</t>
-  </si>
-  <si>
-    <t>.shopping_cart_badge, .btn_inventory</t>
   </si>
   <si>
     <t>Iniciar sesión con credenciales válidas.</t>
@@ -531,7 +564,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="54">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -562,6 +595,7 @@
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
@@ -631,7 +665,7 @@
     <xf borderId="0" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="4" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
@@ -669,6 +703,9 @@
     </xf>
     <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
@@ -998,10 +1035,10 @@
     <col customWidth="1" min="1" max="1" width="5.63"/>
     <col customWidth="1" min="2" max="2" width="39.13"/>
     <col customWidth="1" min="3" max="3" width="9.38"/>
-    <col customWidth="1" min="4" max="4" width="8.63"/>
-    <col customWidth="1" min="5" max="5" width="23.88"/>
+    <col customWidth="1" min="4" max="4" width="13.5"/>
+    <col customWidth="1" min="5" max="5" width="33.13"/>
     <col customWidth="1" min="6" max="6" width="14.38"/>
-    <col customWidth="1" min="7" max="7" width="13.13"/>
+    <col customWidth="1" min="7" max="7" width="19.5"/>
     <col customWidth="1" min="8" max="8" width="15.63"/>
     <col customWidth="1" min="9" max="9" width="4.75"/>
     <col customWidth="1" min="10" max="10" width="38.25"/>
@@ -1503,6 +1540,10 @@
       <c r="AA12" s="3"/>
     </row>
     <row r="13">
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="10"/>
       <c r="I13" s="7">
         <v>3.0</v>
       </c>
@@ -1517,6 +1558,10 @@
       </c>
     </row>
     <row r="14">
+      <c r="C14" s="10"/>
+      <c r="D14" s="10"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="10"/>
       <c r="I14" s="7">
         <v>4.0</v>
       </c>
@@ -1552,7 +1597,7 @@
       <c r="G15" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="H15" s="10">
+      <c r="H15" s="11">
         <v>46053.0</v>
       </c>
       <c r="I15" s="9">
@@ -1569,6 +1614,10 @@
       </c>
     </row>
     <row r="16">
+      <c r="C16" s="10"/>
+      <c r="D16" s="10"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="10"/>
       <c r="I16" s="9">
         <v>2.0</v>
       </c>
@@ -1583,6 +1632,10 @@
       </c>
     </row>
     <row r="17">
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+      <c r="F17" s="10"/>
+      <c r="G17" s="10"/>
       <c r="I17" s="9">
         <v>3.0</v>
       </c>
@@ -1597,6 +1650,10 @@
       </c>
     </row>
     <row r="18">
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="10"/>
       <c r="I18" s="9">
         <v>4.0</v>
       </c>
@@ -2380,6 +2437,10 @@
       <c r="AA37" s="3"/>
     </row>
     <row r="38">
+      <c r="C38" s="10"/>
+      <c r="D38" s="10"/>
+      <c r="F38" s="10"/>
+      <c r="G38" s="10"/>
       <c r="I38" s="9">
         <v>4.0</v>
       </c>
@@ -2394,11 +2455,19 @@
       </c>
     </row>
     <row r="39">
+      <c r="C39" s="10"/>
+      <c r="D39" s="10"/>
+      <c r="F39" s="10"/>
+      <c r="G39" s="10"/>
       <c r="L39" s="1" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="40">
+      <c r="C40" s="10"/>
+      <c r="D40" s="10"/>
+      <c r="F40" s="10"/>
+      <c r="G40" s="10"/>
       <c r="L40" s="1" t="s">
         <v>20</v>
       </c>
@@ -2442,6 +2511,10 @@
       </c>
     </row>
     <row r="42">
+      <c r="C42" s="10"/>
+      <c r="D42" s="10"/>
+      <c r="F42" s="10"/>
+      <c r="G42" s="10"/>
       <c r="I42" s="1">
         <v>2.0</v>
       </c>
@@ -2456,6 +2529,10 @@
       </c>
     </row>
     <row r="43">
+      <c r="C43" s="10"/>
+      <c r="D43" s="10"/>
+      <c r="F43" s="10"/>
+      <c r="G43" s="10"/>
       <c r="I43" s="1">
         <v>3.0</v>
       </c>
@@ -2470,6 +2547,10 @@
       </c>
     </row>
     <row r="44">
+      <c r="C44" s="10"/>
+      <c r="D44" s="10"/>
+      <c r="F44" s="10"/>
+      <c r="G44" s="10"/>
       <c r="I44" s="9">
         <v>4.0</v>
       </c>
@@ -2484,537 +2565,544 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="11" t="s">
+      <c r="A45" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="B45" s="12" t="s">
+      <c r="B45" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="C45" s="12" t="s">
+      <c r="C45" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="D45" s="13" t="s">
+      <c r="D45" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="E45" s="14" t="s">
+      <c r="E45" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="F45" s="13" t="s">
+      <c r="F45" s="14" t="s">
         <v>16</v>
       </c>
       <c r="G45" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="H45" s="15">
+      <c r="H45" s="16">
         <v>46066.0</v>
       </c>
-      <c r="I45" s="16">
+      <c r="I45" s="17">
         <v>1.0</v>
       </c>
-      <c r="J45" s="17" t="s">
+      <c r="J45" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="K45" s="18" t="s">
+      <c r="K45" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="L45" s="13" t="s">
+      <c r="L45" s="14" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="19"/>
-      <c r="B46" s="20"/>
-      <c r="C46" s="20"/>
-      <c r="D46" s="20"/>
-      <c r="F46" s="20"/>
-      <c r="G46" s="20"/>
-      <c r="H46" s="20"/>
-      <c r="I46" s="21">
+      <c r="A46" s="20"/>
+      <c r="B46" s="21"/>
+      <c r="C46" s="21"/>
+      <c r="D46" s="21"/>
+      <c r="F46" s="21"/>
+      <c r="G46" s="21"/>
+      <c r="H46" s="21"/>
+      <c r="I46" s="22">
         <v>2.0</v>
       </c>
-      <c r="J46" s="22" t="s">
+      <c r="J46" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="K46" s="23" t="s">
+      <c r="K46" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="L46" s="22" t="s">
+      <c r="L46" s="23" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="11"/>
-      <c r="B47" s="12"/>
-      <c r="C47" s="12"/>
-      <c r="D47" s="12"/>
-      <c r="F47" s="12"/>
-      <c r="G47" s="12"/>
-      <c r="H47" s="12"/>
-      <c r="I47" s="16">
+      <c r="A47" s="12"/>
+      <c r="B47" s="13"/>
+      <c r="C47" s="13"/>
+      <c r="D47" s="13"/>
+      <c r="F47" s="13"/>
+      <c r="G47" s="13"/>
+      <c r="H47" s="13"/>
+      <c r="I47" s="17">
         <v>3.0</v>
       </c>
-      <c r="J47" s="13" t="s">
+      <c r="J47" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="K47" s="13" t="s">
+      <c r="K47" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="L47" s="13" t="s">
+      <c r="L47" s="14" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="19"/>
-      <c r="B48" s="20"/>
-      <c r="C48" s="20"/>
-      <c r="D48" s="20"/>
-      <c r="F48" s="20"/>
-      <c r="G48" s="20"/>
-      <c r="H48" s="20"/>
-      <c r="I48" s="21">
+      <c r="A48" s="20"/>
+      <c r="B48" s="21"/>
+      <c r="C48" s="21"/>
+      <c r="D48" s="21"/>
+      <c r="F48" s="21"/>
+      <c r="G48" s="21"/>
+      <c r="H48" s="21"/>
+      <c r="I48" s="22">
         <v>4.0</v>
       </c>
-      <c r="J48" s="20" t="s">
+      <c r="J48" s="21" t="s">
         <v>85</v>
       </c>
-      <c r="K48" s="20" t="s">
+      <c r="K48" s="21" t="s">
         <v>86</v>
       </c>
-      <c r="L48" s="22" t="s">
+      <c r="L48" s="23" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="24"/>
-      <c r="B49" s="25"/>
-      <c r="C49" s="25"/>
-      <c r="D49" s="25"/>
-      <c r="F49" s="25"/>
-      <c r="G49" s="25"/>
-      <c r="H49" s="25"/>
-      <c r="I49" s="26">
+      <c r="A49" s="25"/>
+      <c r="B49" s="26"/>
+      <c r="C49" s="26"/>
+      <c r="D49" s="26"/>
+      <c r="F49" s="26"/>
+      <c r="G49" s="26"/>
+      <c r="H49" s="26"/>
+      <c r="I49" s="27">
         <v>5.0</v>
       </c>
-      <c r="J49" s="12" t="s">
+      <c r="J49" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="K49" s="12" t="s">
+      <c r="K49" s="13" t="s">
         <v>88</v>
       </c>
-      <c r="L49" s="13" t="s">
+      <c r="L49" s="14" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="27"/>
-      <c r="B50" s="28"/>
-      <c r="C50" s="28"/>
-      <c r="D50" s="28"/>
-      <c r="F50" s="28"/>
-      <c r="G50" s="28"/>
-      <c r="H50" s="28"/>
-      <c r="I50" s="29">
+      <c r="A50" s="28"/>
+      <c r="B50" s="29"/>
+      <c r="C50" s="29"/>
+      <c r="D50" s="29"/>
+      <c r="F50" s="29"/>
+      <c r="G50" s="29"/>
+      <c r="H50" s="29"/>
+      <c r="I50" s="30">
         <v>6.0</v>
       </c>
-      <c r="J50" s="20" t="s">
+      <c r="J50" s="21" t="s">
         <v>89</v>
       </c>
-      <c r="K50" s="20" t="s">
+      <c r="K50" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="L50" s="22" t="s">
+      <c r="L50" s="23" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="30"/>
-      <c r="B51" s="25"/>
-      <c r="C51" s="25"/>
-      <c r="D51" s="25"/>
-      <c r="E51" s="25"/>
-      <c r="F51" s="25"/>
-      <c r="G51" s="25"/>
-      <c r="H51" s="25"/>
-      <c r="I51" s="24"/>
-      <c r="J51" s="12"/>
-      <c r="K51" s="12"/>
-      <c r="L51" s="12"/>
+      <c r="A51" s="31"/>
+      <c r="B51" s="26"/>
+      <c r="C51" s="26"/>
+      <c r="D51" s="26"/>
+      <c r="E51" s="26"/>
+      <c r="F51" s="26"/>
+      <c r="G51" s="26"/>
+      <c r="H51" s="26"/>
+      <c r="I51" s="25"/>
+      <c r="J51" s="13"/>
+      <c r="K51" s="13"/>
+      <c r="L51" s="13"/>
     </row>
     <row r="52">
-      <c r="A52" s="31" t="s">
+      <c r="A52" s="32" t="s">
         <v>91</v>
       </c>
-      <c r="B52" s="32" t="s">
+      <c r="B52" s="33" t="s">
         <v>92</v>
       </c>
-      <c r="C52" s="32" t="s">
+      <c r="C52" s="33" t="s">
         <v>13</v>
       </c>
-      <c r="D52" s="22" t="s">
+      <c r="D52" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="E52" s="33" t="s">
+      <c r="E52" s="34" t="s">
         <v>93</v>
       </c>
-      <c r="F52" s="22" t="s">
+      <c r="F52" s="23" t="s">
         <v>16</v>
       </c>
       <c r="G52" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="H52" s="34">
+      <c r="H52" s="35">
         <v>46067.0</v>
       </c>
-      <c r="I52" s="29">
+      <c r="I52" s="30">
         <v>1.0</v>
       </c>
-      <c r="J52" s="23" t="s">
+      <c r="J52" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="K52" s="35" t="s">
+      <c r="K52" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="L52" s="22" t="s">
+      <c r="L52" s="23" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="30"/>
-      <c r="B53" s="25"/>
-      <c r="C53" s="36"/>
-      <c r="D53" s="36"/>
-      <c r="F53" s="36"/>
-      <c r="G53" s="36"/>
-      <c r="H53" s="37"/>
-      <c r="I53" s="26">
+      <c r="A53" s="31"/>
+      <c r="B53" s="26"/>
+      <c r="C53" s="37"/>
+      <c r="D53" s="37"/>
+      <c r="F53" s="37"/>
+      <c r="G53" s="37"/>
+      <c r="H53" s="38"/>
+      <c r="I53" s="27">
         <v>2.0</v>
       </c>
-      <c r="J53" s="13" t="s">
+      <c r="J53" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="K53" s="17" t="s">
+      <c r="K53" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="L53" s="13" t="s">
+      <c r="L53" s="14" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="31"/>
-      <c r="B54" s="28"/>
-      <c r="C54" s="32"/>
-      <c r="D54" s="32"/>
-      <c r="F54" s="32"/>
-      <c r="G54" s="32"/>
-      <c r="H54" s="34"/>
-      <c r="I54" s="29">
+      <c r="A54" s="32"/>
+      <c r="B54" s="29"/>
+      <c r="C54" s="33"/>
+      <c r="D54" s="33"/>
+      <c r="F54" s="33"/>
+      <c r="G54" s="33"/>
+      <c r="H54" s="35"/>
+      <c r="I54" s="30">
         <v>3.0</v>
       </c>
-      <c r="J54" s="22" t="s">
+      <c r="J54" s="23" t="s">
         <v>54</v>
       </c>
-      <c r="K54" s="22" t="s">
+      <c r="K54" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="L54" s="22" t="s">
+      <c r="L54" s="23" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="38"/>
-      <c r="B55" s="38"/>
-      <c r="C55" s="38"/>
-      <c r="D55" s="38"/>
-      <c r="E55" s="18"/>
-      <c r="F55" s="38"/>
-      <c r="G55" s="38"/>
-      <c r="H55" s="39"/>
-      <c r="I55" s="40">
+      <c r="A55" s="39"/>
+      <c r="B55" s="39"/>
+      <c r="C55" s="39"/>
+      <c r="D55" s="39"/>
+      <c r="F55" s="39"/>
+      <c r="G55" s="39"/>
+      <c r="H55" s="40"/>
+      <c r="I55" s="41">
         <v>4.0</v>
       </c>
-      <c r="J55" s="38" t="s">
+      <c r="J55" s="39" t="s">
         <v>94</v>
       </c>
-      <c r="K55" s="38" t="s">
+      <c r="K55" s="39" t="s">
         <v>95</v>
       </c>
-      <c r="L55" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="M55" s="41"/>
-      <c r="N55" s="41"/>
-      <c r="O55" s="41"/>
-      <c r="P55" s="41"/>
-      <c r="Q55" s="41"/>
-      <c r="R55" s="41"/>
-      <c r="S55" s="41"/>
-      <c r="T55" s="41"/>
-      <c r="U55" s="41"/>
-      <c r="V55" s="41"/>
-      <c r="W55" s="41"/>
-      <c r="X55" s="41"/>
-      <c r="Y55" s="41"/>
-      <c r="Z55" s="41"/>
-      <c r="AA55" s="41"/>
+      <c r="L55" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="M55" s="42"/>
+      <c r="N55" s="42"/>
+      <c r="O55" s="42"/>
+      <c r="P55" s="42"/>
+      <c r="Q55" s="42"/>
+      <c r="R55" s="42"/>
+      <c r="S55" s="42"/>
+      <c r="T55" s="42"/>
+      <c r="U55" s="42"/>
+      <c r="V55" s="42"/>
+      <c r="W55" s="42"/>
+      <c r="X55" s="42"/>
+      <c r="Y55" s="42"/>
+      <c r="Z55" s="42"/>
+      <c r="AA55" s="42"/>
     </row>
     <row r="56">
-      <c r="A56" s="42"/>
-      <c r="B56" s="42"/>
-      <c r="C56" s="42"/>
-      <c r="D56" s="42"/>
-      <c r="E56" s="35"/>
-      <c r="F56" s="42"/>
-      <c r="G56" s="42"/>
-      <c r="H56" s="43"/>
-      <c r="I56" s="44">
+      <c r="A56" s="43"/>
+      <c r="B56" s="43"/>
+      <c r="C56" s="43"/>
+      <c r="D56" s="43"/>
+      <c r="F56" s="43"/>
+      <c r="G56" s="43"/>
+      <c r="H56" s="44"/>
+      <c r="I56" s="45">
         <v>5.0</v>
       </c>
-      <c r="J56" s="42" t="s">
+      <c r="J56" s="43" t="s">
         <v>96</v>
       </c>
-      <c r="K56" s="42" t="s">
+      <c r="K56" s="43" t="s">
         <v>97</v>
       </c>
-      <c r="L56" s="22" t="s">
-        <v>20</v>
-      </c>
-      <c r="M56" s="41"/>
-      <c r="N56" s="41"/>
-      <c r="O56" s="41"/>
-      <c r="P56" s="41"/>
-      <c r="Q56" s="41"/>
-      <c r="R56" s="41"/>
-      <c r="S56" s="41"/>
-      <c r="T56" s="41"/>
-      <c r="U56" s="41"/>
-      <c r="V56" s="41"/>
-      <c r="W56" s="41"/>
-      <c r="X56" s="41"/>
-      <c r="Y56" s="41"/>
-      <c r="Z56" s="41"/>
-      <c r="AA56" s="41"/>
+      <c r="L56" s="23" t="s">
+        <v>20</v>
+      </c>
+      <c r="M56" s="42"/>
+      <c r="N56" s="42"/>
+      <c r="O56" s="42"/>
+      <c r="P56" s="42"/>
+      <c r="Q56" s="42"/>
+      <c r="R56" s="42"/>
+      <c r="S56" s="42"/>
+      <c r="T56" s="42"/>
+      <c r="U56" s="42"/>
+      <c r="V56" s="42"/>
+      <c r="W56" s="42"/>
+      <c r="X56" s="42"/>
+      <c r="Y56" s="42"/>
+      <c r="Z56" s="42"/>
+      <c r="AA56" s="42"/>
     </row>
     <row r="57">
-      <c r="A57" s="38"/>
-      <c r="B57" s="38"/>
-      <c r="C57" s="38"/>
-      <c r="D57" s="38"/>
-      <c r="E57" s="18"/>
-      <c r="F57" s="38"/>
-      <c r="G57" s="38"/>
-      <c r="H57" s="39"/>
-      <c r="I57" s="40">
+      <c r="A57" s="39"/>
+      <c r="B57" s="39"/>
+      <c r="C57" s="39"/>
+      <c r="D57" s="39"/>
+      <c r="F57" s="39"/>
+      <c r="G57" s="39"/>
+      <c r="H57" s="40"/>
+      <c r="I57" s="41">
         <v>6.0</v>
       </c>
-      <c r="J57" s="38" t="s">
+      <c r="J57" s="39" t="s">
         <v>98</v>
       </c>
-      <c r="K57" s="38" t="s">
+      <c r="K57" s="39" t="s">
         <v>99</v>
       </c>
-      <c r="L57" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="M57" s="41"/>
-      <c r="N57" s="41"/>
-      <c r="O57" s="41"/>
-      <c r="P57" s="41"/>
-      <c r="Q57" s="41"/>
-      <c r="R57" s="41"/>
-      <c r="S57" s="41"/>
-      <c r="T57" s="41"/>
-      <c r="U57" s="41"/>
-      <c r="V57" s="41"/>
-      <c r="W57" s="41"/>
-      <c r="X57" s="41"/>
-      <c r="Y57" s="41"/>
-      <c r="Z57" s="41"/>
-      <c r="AA57" s="41"/>
+      <c r="L57" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="M57" s="42"/>
+      <c r="N57" s="42"/>
+      <c r="O57" s="42"/>
+      <c r="P57" s="42"/>
+      <c r="Q57" s="42"/>
+      <c r="R57" s="42"/>
+      <c r="S57" s="42"/>
+      <c r="T57" s="42"/>
+      <c r="U57" s="42"/>
+      <c r="V57" s="42"/>
+      <c r="W57" s="42"/>
+      <c r="X57" s="42"/>
+      <c r="Y57" s="42"/>
+      <c r="Z57" s="42"/>
+      <c r="AA57" s="42"/>
     </row>
     <row r="58">
-      <c r="A58" s="42"/>
-      <c r="B58" s="42"/>
-      <c r="C58" s="42"/>
-      <c r="D58" s="42"/>
-      <c r="E58" s="35"/>
-      <c r="F58" s="42"/>
-      <c r="G58" s="42"/>
-      <c r="H58" s="43"/>
-      <c r="I58" s="42"/>
-      <c r="J58" s="42"/>
-      <c r="K58" s="42"/>
-      <c r="L58" s="42"/>
-      <c r="M58" s="41"/>
-      <c r="N58" s="41"/>
-      <c r="O58" s="41"/>
-      <c r="P58" s="41"/>
-      <c r="Q58" s="41"/>
-      <c r="R58" s="41"/>
-      <c r="S58" s="41"/>
-      <c r="T58" s="41"/>
-      <c r="U58" s="41"/>
-      <c r="V58" s="41"/>
-      <c r="W58" s="41"/>
-      <c r="X58" s="41"/>
-      <c r="Y58" s="41"/>
-      <c r="Z58" s="41"/>
-      <c r="AA58" s="41"/>
+      <c r="A58" s="43"/>
+      <c r="B58" s="43"/>
+      <c r="C58" s="43"/>
+      <c r="D58" s="43"/>
+      <c r="F58" s="43"/>
+      <c r="G58" s="43"/>
+      <c r="H58" s="44"/>
+      <c r="I58" s="43"/>
+      <c r="J58" s="43"/>
+      <c r="K58" s="43"/>
+      <c r="L58" s="43"/>
+      <c r="M58" s="42"/>
+      <c r="N58" s="42"/>
+      <c r="O58" s="42"/>
+      <c r="P58" s="42"/>
+      <c r="Q58" s="42"/>
+      <c r="R58" s="42"/>
+      <c r="S58" s="42"/>
+      <c r="T58" s="42"/>
+      <c r="U58" s="42"/>
+      <c r="V58" s="42"/>
+      <c r="W58" s="42"/>
+      <c r="X58" s="42"/>
+      <c r="Y58" s="42"/>
+      <c r="Z58" s="42"/>
+      <c r="AA58" s="42"/>
     </row>
     <row r="59">
-      <c r="A59" s="30" t="s">
+      <c r="A59" s="14" t="s">
         <v>100</v>
       </c>
-      <c r="B59" s="36" t="s">
+      <c r="B59" s="46" t="s">
         <v>101</v>
       </c>
-      <c r="C59" s="36" t="s">
+      <c r="C59" s="46" t="s">
         <v>13</v>
       </c>
-      <c r="D59" s="36" t="s">
+      <c r="D59" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="E59" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="E59" s="45" t="s">
+      <c r="F59" s="18" t="s">
         <v>103</v>
       </c>
-      <c r="F59" s="36" t="s">
+      <c r="G59" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H59" s="46" t="s">
         <v>104</v>
       </c>
-      <c r="G59" s="36" t="s">
+      <c r="I59" s="47">
+        <v>1.0</v>
+      </c>
+      <c r="J59" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="K59" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="L59" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="M59" s="3"/>
+      <c r="N59" s="3"/>
+      <c r="O59" s="3"/>
+      <c r="P59" s="3"/>
+      <c r="Q59" s="3"/>
+      <c r="R59" s="3"/>
+      <c r="S59" s="3"/>
+      <c r="T59" s="3"/>
+      <c r="U59" s="3"/>
+      <c r="V59" s="3"/>
+      <c r="W59" s="3"/>
+      <c r="X59" s="3"/>
+      <c r="Y59" s="3"/>
+      <c r="Z59" s="3"/>
+      <c r="AA59" s="3"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="32"/>
+      <c r="B60" s="29"/>
+      <c r="C60" s="33"/>
+      <c r="D60" s="33"/>
+      <c r="F60" s="33"/>
+      <c r="G60" s="33"/>
+      <c r="H60" s="35"/>
+      <c r="I60" s="30">
+        <v>2.0</v>
+      </c>
+      <c r="J60" s="23" t="s">
+        <v>46</v>
+      </c>
+      <c r="K60" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="L60" s="45" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="31"/>
+      <c r="B61" s="26"/>
+      <c r="C61" s="37"/>
+      <c r="D61" s="37"/>
+      <c r="F61" s="37"/>
+      <c r="G61" s="37"/>
+      <c r="H61" s="38"/>
+      <c r="I61" s="27">
+        <v>3.0</v>
+      </c>
+      <c r="J61" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="K61" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="L61" s="41" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="28"/>
+      <c r="B62" s="29"/>
+      <c r="C62" s="29"/>
+      <c r="D62" s="29"/>
+      <c r="F62" s="29"/>
+      <c r="G62" s="29"/>
+      <c r="H62" s="29"/>
+      <c r="I62" s="30">
+        <v>4.0</v>
+      </c>
+      <c r="J62" s="43" t="s">
         <v>105</v>
       </c>
-      <c r="H59" s="37">
-        <v>46069.0</v>
-      </c>
-      <c r="I59" s="26">
-        <v>1.0</v>
-      </c>
-      <c r="J59" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="K59" s="18" t="s">
-        <v>19</v>
-      </c>
-      <c r="L59" s="38" t="s">
+      <c r="K62" s="43" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="31"/>
-      <c r="B60" s="28"/>
-      <c r="C60" s="32"/>
-      <c r="D60" s="32"/>
-      <c r="E60" s="28"/>
-      <c r="F60" s="32"/>
-      <c r="G60" s="32"/>
-      <c r="H60" s="34"/>
-      <c r="I60" s="29">
-        <v>2.0</v>
-      </c>
-      <c r="J60" s="22" t="s">
-        <v>46</v>
-      </c>
-      <c r="K60" s="23" t="s">
-        <v>22</v>
-      </c>
-      <c r="L60" s="42" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="30"/>
-      <c r="B61" s="25"/>
-      <c r="C61" s="36"/>
-      <c r="D61" s="36"/>
-      <c r="E61" s="25"/>
-      <c r="F61" s="36"/>
-      <c r="G61" s="36"/>
-      <c r="H61" s="37"/>
-      <c r="I61" s="26">
-        <v>3.0</v>
-      </c>
-      <c r="J61" s="13" t="s">
-        <v>54</v>
-      </c>
-      <c r="K61" s="13" t="s">
-        <v>55</v>
-      </c>
-      <c r="L61" s="38" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="27"/>
-      <c r="B62" s="28"/>
-      <c r="C62" s="28"/>
-      <c r="D62" s="28"/>
-      <c r="E62" s="28"/>
-      <c r="F62" s="28"/>
-      <c r="G62" s="28"/>
-      <c r="H62" s="28"/>
-      <c r="I62" s="29">
-        <v>4.0</v>
-      </c>
-      <c r="J62" s="42" t="s">
+      <c r="L62" s="45" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="25"/>
+      <c r="B63" s="26"/>
+      <c r="C63" s="26"/>
+      <c r="D63" s="26"/>
+      <c r="F63" s="26"/>
+      <c r="G63" s="26"/>
+      <c r="H63" s="26"/>
+      <c r="I63" s="27">
+        <v>5.0</v>
+      </c>
+      <c r="J63" s="39" t="s">
         <v>107</v>
       </c>
-      <c r="K62" s="42" t="s">
+      <c r="K63" s="39" t="s">
         <v>108</v>
       </c>
-      <c r="L62" s="42" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="24"/>
-      <c r="B63" s="25"/>
-      <c r="C63" s="25"/>
-      <c r="D63" s="25"/>
-      <c r="E63" s="25"/>
-      <c r="F63" s="25"/>
-      <c r="G63" s="25"/>
-      <c r="H63" s="25"/>
-      <c r="I63" s="26">
-        <v>5.0</v>
-      </c>
-      <c r="J63" s="38" t="s">
+      <c r="L63" s="41" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="64" ht="39.0" customHeight="1">
+      <c r="A64" s="28"/>
+      <c r="B64" s="29"/>
+      <c r="C64" s="29"/>
+      <c r="D64" s="29"/>
+      <c r="F64" s="29"/>
+      <c r="G64" s="29"/>
+      <c r="H64" s="29"/>
+      <c r="I64" s="30">
+        <v>6.0</v>
+      </c>
+      <c r="J64" s="43" t="s">
         <v>109</v>
       </c>
-      <c r="K63" s="38" t="s">
+      <c r="K64" s="43" t="s">
         <v>110</v>
       </c>
-      <c r="L63" s="38" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="27"/>
-      <c r="B64" s="28"/>
-      <c r="C64" s="28"/>
-      <c r="D64" s="28"/>
-      <c r="E64" s="28"/>
-      <c r="F64" s="28"/>
-      <c r="G64" s="28"/>
-      <c r="H64" s="28"/>
-      <c r="I64" s="29">
-        <v>6.0</v>
-      </c>
-      <c r="J64" s="42" t="s">
-        <v>111</v>
-      </c>
-      <c r="K64" s="42" t="s">
-        <v>112</v>
-      </c>
-      <c r="L64" s="42" t="s">
-        <v>106</v>
+      <c r="L64" s="45" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="13">
     <mergeCell ref="E31:E34"/>
     <mergeCell ref="E35:E39"/>
     <mergeCell ref="E41:E44"/>
     <mergeCell ref="E45:E50"/>
-    <mergeCell ref="E52:E54"/>
+    <mergeCell ref="E52:E58"/>
+    <mergeCell ref="E59:E64"/>
     <mergeCell ref="E2:E6"/>
     <mergeCell ref="E7:E10"/>
     <mergeCell ref="E11:E14"/>
@@ -3023,6 +3111,23 @@
     <mergeCell ref="E23:E26"/>
     <mergeCell ref="E27:E30"/>
   </mergeCells>
+  <dataValidations>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:C59">
+      <formula1>"P0 (Crítica),P0"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="D2:D57 D59">
+      <formula1>"Finalizado,Pendiente"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="G2:G57 G59">
+      <formula1>"PENDIENTE 🟡,PASSED 🟢"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="F2:F57 F59">
+      <formula1>"❌ NO PENDIENTE 🟡,✅ SÍ (Playwright) PASSED 🟢"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="L2:L64">
+      <formula1>"Hecho,Pending"</formula1>
+    </dataValidation>
+  </dataValidations>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
@@ -3036,10 +3141,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="9" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2">
@@ -3069,145 +3174,145 @@
   </cols>
   <sheetData>
     <row r="45" ht="22.5" customHeight="1">
-      <c r="A45" s="46" t="s">
+      <c r="A45" s="48" t="s">
         <v>0</v>
       </c>
-      <c r="B45" s="47" t="s">
+      <c r="B45" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="C45" s="47" t="s">
+      <c r="C45" s="49" t="s">
         <v>2</v>
       </c>
-      <c r="D45" s="47" t="s">
+      <c r="D45" s="49" t="s">
         <v>3</v>
       </c>
-      <c r="E45" s="47" t="s">
+      <c r="E45" s="49" t="s">
         <v>4</v>
       </c>
-      <c r="F45" s="47" t="s">
+      <c r="F45" s="49" t="s">
         <v>5</v>
       </c>
-      <c r="G45" s="47" t="s">
+      <c r="G45" s="49" t="s">
         <v>6</v>
       </c>
-      <c r="H45" s="47" t="s">
+      <c r="H45" s="49" t="s">
         <v>7</v>
       </c>
-      <c r="I45" s="46" t="s">
+      <c r="I45" s="48" t="s">
         <v>8</v>
       </c>
-      <c r="J45" s="47" t="s">
+      <c r="J45" s="49" t="s">
         <v>9</v>
       </c>
-      <c r="K45" s="47" t="s">
+      <c r="K45" s="49" t="s">
         <v>10</v>
       </c>
-      <c r="L45" s="47" t="s">
+      <c r="L45" s="49" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="46" ht="22.5" customHeight="1">
+      <c r="A46" s="50" t="s">
+        <v>82</v>
+      </c>
+      <c r="B46" s="51" t="s">
+        <v>83</v>
+      </c>
+      <c r="C46" s="51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D46" s="51" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="46" ht="22.5" customHeight="1">
-      <c r="A46" s="48" t="s">
-        <v>82</v>
-      </c>
-      <c r="B46" s="49" t="s">
-        <v>83</v>
-      </c>
-      <c r="C46" s="49" t="s">
-        <v>13</v>
-      </c>
-      <c r="D46" s="49" t="s">
-        <v>102</v>
-      </c>
-      <c r="E46" s="49" t="s">
+      <c r="E46" s="51" t="s">
         <v>115</v>
       </c>
-      <c r="F46" s="49" t="s">
-        <v>104</v>
-      </c>
-      <c r="G46" s="49" t="s">
-        <v>105</v>
-      </c>
-      <c r="H46" s="50">
+      <c r="F46" s="51" t="s">
+        <v>111</v>
+      </c>
+      <c r="G46" s="51" t="s">
+        <v>116</v>
+      </c>
+      <c r="H46" s="52">
         <v>46066.0</v>
       </c>
-      <c r="I46" s="51">
+      <c r="I46" s="53">
         <v>1.0</v>
       </c>
-      <c r="J46" s="49" t="s">
-        <v>116</v>
-      </c>
-      <c r="K46" s="49" t="s">
+      <c r="J46" s="51" t="s">
         <v>117</v>
       </c>
-      <c r="L46" s="49" t="s">
-        <v>102</v>
+      <c r="K46" s="51" t="s">
+        <v>118</v>
+      </c>
+      <c r="L46" s="51" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="47" ht="22.5" customHeight="1">
-      <c r="A47" s="48"/>
-      <c r="B47" s="49"/>
-      <c r="C47" s="49"/>
-      <c r="D47" s="49"/>
-      <c r="E47" s="49"/>
-      <c r="F47" s="49"/>
-      <c r="G47" s="49"/>
-      <c r="H47" s="49"/>
-      <c r="I47" s="51">
+      <c r="A47" s="50"/>
+      <c r="B47" s="51"/>
+      <c r="C47" s="51"/>
+      <c r="D47" s="51"/>
+      <c r="E47" s="51"/>
+      <c r="F47" s="51"/>
+      <c r="G47" s="51"/>
+      <c r="H47" s="51"/>
+      <c r="I47" s="53">
         <v>2.0</v>
       </c>
-      <c r="J47" s="49" t="s">
+      <c r="J47" s="51" t="s">
         <v>85</v>
       </c>
-      <c r="K47" s="49" t="s">
+      <c r="K47" s="51" t="s">
         <v>86</v>
       </c>
-      <c r="L47" s="49" t="s">
-        <v>102</v>
+      <c r="L47" s="51" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="48" ht="22.5" customHeight="1">
-      <c r="A48" s="48"/>
-      <c r="B48" s="49"/>
-      <c r="C48" s="49"/>
-      <c r="D48" s="49"/>
-      <c r="E48" s="49"/>
-      <c r="F48" s="49"/>
-      <c r="G48" s="49"/>
-      <c r="H48" s="49"/>
-      <c r="I48" s="51">
+      <c r="A48" s="50"/>
+      <c r="B48" s="51"/>
+      <c r="C48" s="51"/>
+      <c r="D48" s="51"/>
+      <c r="E48" s="51"/>
+      <c r="F48" s="51"/>
+      <c r="G48" s="51"/>
+      <c r="H48" s="51"/>
+      <c r="I48" s="53">
         <v>3.0</v>
       </c>
-      <c r="J48" s="49" t="s">
+      <c r="J48" s="51" t="s">
         <v>87</v>
       </c>
-      <c r="K48" s="49" t="s">
+      <c r="K48" s="51" t="s">
         <v>88</v>
       </c>
-      <c r="L48" s="49" t="s">
-        <v>102</v>
+      <c r="L48" s="51" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="49" ht="22.5" customHeight="1">
-      <c r="A49" s="48"/>
-      <c r="B49" s="49"/>
-      <c r="C49" s="49"/>
-      <c r="D49" s="49"/>
-      <c r="E49" s="49"/>
-      <c r="F49" s="49"/>
-      <c r="G49" s="49"/>
-      <c r="H49" s="49"/>
-      <c r="I49" s="51">
+      <c r="A49" s="50"/>
+      <c r="B49" s="51"/>
+      <c r="C49" s="51"/>
+      <c r="D49" s="51"/>
+      <c r="E49" s="51"/>
+      <c r="F49" s="51"/>
+      <c r="G49" s="51"/>
+      <c r="H49" s="51"/>
+      <c r="I49" s="53">
         <v>4.0</v>
       </c>
-      <c r="J49" s="49" t="s">
+      <c r="J49" s="51" t="s">
         <v>89</v>
       </c>
-      <c r="K49" s="49" t="s">
+      <c r="K49" s="51" t="s">
         <v>90</v>
       </c>
-      <c r="L49" s="49" t="s">
-        <v>102</v>
+      <c r="L49" s="51" t="s">
+        <v>114</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: Update dashboard for Session 12 with roadmap and conversion focus
</commit_message>
<xml_diff>
--- a/docs/QA_Roadmap_Natalia.xlsx
+++ b/docs/QA_Roadmap_Natalia.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="123">
   <si>
     <t>ID</t>
   </si>
@@ -477,6 +477,39 @@
     <t>The badge decreases or disappears.</t>
   </si>
   <si>
+    <t>TC-14</t>
+  </si>
+  <si>
+    <t>Verificar la efectiva cancelacion del checkout.</t>
+  </si>
+  <si>
+    <t>Pendiente</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <b val="0"/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">[data-test="login-button"], [data-test="username"], [data-test="password"], .inventory_list, .inventory_item, .title, .shopping_cart_badge, .btn_inventory., shopping_cart_link, .inventory_item_name, .cart_item, '[data-test="continue-shopping"]', </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <b/>
+        <color theme="1"/>
+      </rPr>
+      <t>.cart_cancel_link</t>
+    </r>
+  </si>
+  <si>
+    <t>❌ NO PENDIENTE 🟡</t>
+  </si>
+  <si>
+    <t>PENDIENTE 🟡</t>
+  </si>
+  <si>
     <t>❌ NO</t>
   </si>
   <si>
@@ -486,13 +519,7 @@
     <t>Estado 2</t>
   </si>
   <si>
-    <t>Pendiente</t>
-  </si>
-  <si>
     <t>.shopping_cart_badge, .btn_inventory</t>
-  </si>
-  <si>
-    <t>PENDIENTE 🟡</t>
   </si>
   <si>
     <t>Iniciar sesión con credenciales válidas.</t>
@@ -564,7 +591,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="68">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -706,6 +733,48 @@
     </xf>
     <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="top"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="top"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="top"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="top"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
@@ -3095,14 +3164,121 @@
         <v>20</v>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" s="27" t="s">
+        <v>111</v>
+      </c>
+      <c r="B65" s="37" t="s">
+        <v>112</v>
+      </c>
+      <c r="C65" s="46" t="s">
+        <v>65</v>
+      </c>
+      <c r="D65" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="E65" s="15" t="s">
+        <v>114</v>
+      </c>
+      <c r="F65" s="18" t="s">
+        <v>115</v>
+      </c>
+      <c r="G65" s="18" t="s">
+        <v>116</v>
+      </c>
+      <c r="H65" s="38">
+        <v>45346.0</v>
+      </c>
+      <c r="I65" s="27">
+        <v>1.0</v>
+      </c>
+      <c r="J65" s="41"/>
+      <c r="K65" s="41"/>
+      <c r="L65" s="48"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="49"/>
+      <c r="B66" s="50"/>
+      <c r="C66" s="51"/>
+      <c r="D66" s="52"/>
+      <c r="F66" s="52"/>
+      <c r="G66" s="53"/>
+      <c r="H66" s="50"/>
+      <c r="I66" s="30">
+        <v>2.0</v>
+      </c>
+      <c r="J66" s="45"/>
+      <c r="K66" s="45"/>
+      <c r="L66" s="54"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="55"/>
+      <c r="B67" s="56"/>
+      <c r="C67" s="57"/>
+      <c r="D67" s="58"/>
+      <c r="F67" s="58"/>
+      <c r="G67" s="59"/>
+      <c r="H67" s="56"/>
+      <c r="I67" s="27">
+        <v>3.0</v>
+      </c>
+      <c r="J67" s="41"/>
+      <c r="K67" s="41"/>
+      <c r="L67" s="48"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="49"/>
+      <c r="B68" s="50"/>
+      <c r="C68" s="51"/>
+      <c r="D68" s="52"/>
+      <c r="F68" s="52"/>
+      <c r="G68" s="53"/>
+      <c r="H68" s="50"/>
+      <c r="I68" s="30">
+        <v>4.0</v>
+      </c>
+      <c r="J68" s="45"/>
+      <c r="K68" s="45"/>
+      <c r="L68" s="54"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="55"/>
+      <c r="B69" s="56"/>
+      <c r="C69" s="57"/>
+      <c r="D69" s="58"/>
+      <c r="F69" s="58"/>
+      <c r="G69" s="59"/>
+      <c r="H69" s="56"/>
+      <c r="I69" s="27">
+        <v>5.0</v>
+      </c>
+      <c r="J69" s="41"/>
+      <c r="K69" s="41"/>
+      <c r="L69" s="48"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="49"/>
+      <c r="B70" s="50"/>
+      <c r="C70" s="51"/>
+      <c r="D70" s="52"/>
+      <c r="E70" s="60"/>
+      <c r="F70" s="52"/>
+      <c r="G70" s="53"/>
+      <c r="H70" s="50"/>
+      <c r="I70" s="30"/>
+      <c r="J70" s="61"/>
+      <c r="K70" s="61"/>
+      <c r="L70" s="54"/>
+    </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="14">
     <mergeCell ref="E31:E34"/>
     <mergeCell ref="E35:E39"/>
     <mergeCell ref="E41:E44"/>
     <mergeCell ref="E45:E50"/>
     <mergeCell ref="E52:E58"/>
     <mergeCell ref="E59:E64"/>
+    <mergeCell ref="E65:E69"/>
     <mergeCell ref="E2:E6"/>
     <mergeCell ref="E7:E10"/>
     <mergeCell ref="E11:E14"/>
@@ -3112,16 +3288,16 @@
     <mergeCell ref="E27:E30"/>
   </mergeCells>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:C59">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:C59 C65">
       <formula1>"P0 (Crítica),P0"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="D2:D57 D59">
+    <dataValidation type="list" allowBlank="1" sqref="D2:D57 D59 D65">
       <formula1>"Finalizado,Pendiente"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="G2:G57 G59">
+    <dataValidation type="list" allowBlank="1" sqref="G2:G57 G59 G65">
       <formula1>"PENDIENTE 🟡,PASSED 🟢"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="F2:F57 F59">
+    <dataValidation type="list" allowBlank="1" sqref="F2:F57 F59 F65">
       <formula1>"❌ NO PENDIENTE 🟡,✅ SÍ (Playwright) PASSED 🟢"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="L2:L64">
@@ -3141,10 +3317,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="9" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
     </row>
     <row r="2">
@@ -3174,145 +3350,145 @@
   </cols>
   <sheetData>
     <row r="45" ht="22.5" customHeight="1">
-      <c r="A45" s="48" t="s">
+      <c r="A45" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="B45" s="49" t="s">
+      <c r="B45" s="63" t="s">
         <v>1</v>
       </c>
-      <c r="C45" s="49" t="s">
+      <c r="C45" s="63" t="s">
         <v>2</v>
       </c>
-      <c r="D45" s="49" t="s">
+      <c r="D45" s="63" t="s">
         <v>3</v>
       </c>
-      <c r="E45" s="49" t="s">
+      <c r="E45" s="63" t="s">
         <v>4</v>
       </c>
-      <c r="F45" s="49" t="s">
+      <c r="F45" s="63" t="s">
         <v>5</v>
       </c>
-      <c r="G45" s="49" t="s">
+      <c r="G45" s="63" t="s">
         <v>6</v>
       </c>
-      <c r="H45" s="49" t="s">
+      <c r="H45" s="63" t="s">
         <v>7</v>
       </c>
-      <c r="I45" s="48" t="s">
+      <c r="I45" s="62" t="s">
         <v>8</v>
       </c>
-      <c r="J45" s="49" t="s">
+      <c r="J45" s="63" t="s">
         <v>9</v>
       </c>
-      <c r="K45" s="49" t="s">
+      <c r="K45" s="63" t="s">
         <v>10</v>
       </c>
-      <c r="L45" s="49" t="s">
+      <c r="L45" s="63" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="46" ht="22.5" customHeight="1">
+      <c r="A46" s="64" t="s">
+        <v>82</v>
+      </c>
+      <c r="B46" s="65" t="s">
+        <v>83</v>
+      </c>
+      <c r="C46" s="65" t="s">
+        <v>13</v>
+      </c>
+      <c r="D46" s="65" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="46" ht="22.5" customHeight="1">
-      <c r="A46" s="50" t="s">
-        <v>82</v>
-      </c>
-      <c r="B46" s="51" t="s">
-        <v>83</v>
-      </c>
-      <c r="C46" s="51" t="s">
-        <v>13</v>
-      </c>
-      <c r="D46" s="51" t="s">
-        <v>114</v>
-      </c>
-      <c r="E46" s="51" t="s">
-        <v>115</v>
-      </c>
-      <c r="F46" s="51" t="s">
-        <v>111</v>
-      </c>
-      <c r="G46" s="51" t="s">
+      <c r="E46" s="65" t="s">
+        <v>120</v>
+      </c>
+      <c r="F46" s="65" t="s">
+        <v>117</v>
+      </c>
+      <c r="G46" s="65" t="s">
         <v>116</v>
       </c>
-      <c r="H46" s="52">
+      <c r="H46" s="66">
         <v>46066.0</v>
       </c>
-      <c r="I46" s="53">
+      <c r="I46" s="67">
         <v>1.0</v>
       </c>
-      <c r="J46" s="51" t="s">
-        <v>117</v>
-      </c>
-      <c r="K46" s="51" t="s">
-        <v>118</v>
-      </c>
-      <c r="L46" s="51" t="s">
-        <v>114</v>
+      <c r="J46" s="65" t="s">
+        <v>121</v>
+      </c>
+      <c r="K46" s="65" t="s">
+        <v>122</v>
+      </c>
+      <c r="L46" s="65" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="47" ht="22.5" customHeight="1">
-      <c r="A47" s="50"/>
-      <c r="B47" s="51"/>
-      <c r="C47" s="51"/>
-      <c r="D47" s="51"/>
-      <c r="E47" s="51"/>
-      <c r="F47" s="51"/>
-      <c r="G47" s="51"/>
-      <c r="H47" s="51"/>
-      <c r="I47" s="53">
+      <c r="A47" s="64"/>
+      <c r="B47" s="65"/>
+      <c r="C47" s="65"/>
+      <c r="D47" s="65"/>
+      <c r="E47" s="65"/>
+      <c r="F47" s="65"/>
+      <c r="G47" s="65"/>
+      <c r="H47" s="65"/>
+      <c r="I47" s="67">
         <v>2.0</v>
       </c>
-      <c r="J47" s="51" t="s">
+      <c r="J47" s="65" t="s">
         <v>85</v>
       </c>
-      <c r="K47" s="51" t="s">
+      <c r="K47" s="65" t="s">
         <v>86</v>
       </c>
-      <c r="L47" s="51" t="s">
-        <v>114</v>
+      <c r="L47" s="65" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="48" ht="22.5" customHeight="1">
-      <c r="A48" s="50"/>
-      <c r="B48" s="51"/>
-      <c r="C48" s="51"/>
-      <c r="D48" s="51"/>
-      <c r="E48" s="51"/>
-      <c r="F48" s="51"/>
-      <c r="G48" s="51"/>
-      <c r="H48" s="51"/>
-      <c r="I48" s="53">
+      <c r="A48" s="64"/>
+      <c r="B48" s="65"/>
+      <c r="C48" s="65"/>
+      <c r="D48" s="65"/>
+      <c r="E48" s="65"/>
+      <c r="F48" s="65"/>
+      <c r="G48" s="65"/>
+      <c r="H48" s="65"/>
+      <c r="I48" s="67">
         <v>3.0</v>
       </c>
-      <c r="J48" s="51" t="s">
+      <c r="J48" s="65" t="s">
         <v>87</v>
       </c>
-      <c r="K48" s="51" t="s">
+      <c r="K48" s="65" t="s">
         <v>88</v>
       </c>
-      <c r="L48" s="51" t="s">
-        <v>114</v>
+      <c r="L48" s="65" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="49" ht="22.5" customHeight="1">
-      <c r="A49" s="50"/>
-      <c r="B49" s="51"/>
-      <c r="C49" s="51"/>
-      <c r="D49" s="51"/>
-      <c r="E49" s="51"/>
-      <c r="F49" s="51"/>
-      <c r="G49" s="51"/>
-      <c r="H49" s="51"/>
-      <c r="I49" s="53">
+      <c r="A49" s="64"/>
+      <c r="B49" s="65"/>
+      <c r="C49" s="65"/>
+      <c r="D49" s="65"/>
+      <c r="E49" s="65"/>
+      <c r="F49" s="65"/>
+      <c r="G49" s="65"/>
+      <c r="H49" s="65"/>
+      <c r="I49" s="67">
         <v>4.0</v>
       </c>
-      <c r="J49" s="51" t="s">
+      <c r="J49" s="65" t="s">
         <v>89</v>
       </c>
-      <c r="K49" s="51" t="s">
+      <c r="K49" s="65" t="s">
         <v>90</v>
       </c>
-      <c r="L49" s="51" t="s">
-        <v>114</v>
+      <c r="L49" s="65" t="s">
+        <v>113</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: Update QA Roadmap document with latest changes and create new explanations.
</commit_message>
<xml_diff>
--- a/docs/QA_Roadmap_Natalia.xlsx
+++ b/docs/QA_Roadmap_Natalia.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="130">
   <si>
     <t>ID</t>
   </si>
@@ -483,9 +483,6 @@
     <t>Verificar la efectiva cancelacion del checkout.</t>
   </si>
   <si>
-    <t>Pendiente</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <rFont val="Arial"/>
@@ -504,22 +501,46 @@
     </r>
   </si>
   <si>
-    <t>❌ NO PENDIENTE 🟡</t>
+    <t>Iniciar sesión y agregar producto al carrito.</t>
+  </si>
+  <si>
+    <t>Página de productos cargada y badge en "1".</t>
+  </si>
+  <si>
+    <t>Navegar al carrito y clic en "Checkout".</t>
+  </si>
+  <si>
+    <t>URL cambia a checkout-step-one.html.</t>
+  </si>
+  <si>
+    <t>Clic en el botón "Cancel".</t>
+  </si>
+  <si>
+    <t>Redirección exitosa a cart.html.</t>
+  </si>
+  <si>
+    <t>Validar estado del carrito.</t>
+  </si>
+  <si>
+    <t>El producto NO se eliminó y el badge sigue en "1".</t>
+  </si>
+  <si>
+    <t>❌ NO</t>
+  </si>
+  <si>
+    <t>PENDIENTE 🟡,</t>
+  </si>
+  <si>
+    <t>Estado 2</t>
+  </si>
+  <si>
+    <t>Pendiente</t>
+  </si>
+  <si>
+    <t>.shopping_cart_badge, .btn_inventory</t>
   </si>
   <si>
     <t>PENDIENTE 🟡</t>
-  </si>
-  <si>
-    <t>❌ NO</t>
-  </si>
-  <si>
-    <t>PENDIENTE 🟡,</t>
-  </si>
-  <si>
-    <t>Estado 2</t>
-  </si>
-  <si>
-    <t>.shopping_cart_badge, .btn_inventory</t>
   </si>
   <si>
     <t>Iniciar sesión con credenciales válidas.</t>
@@ -591,7 +612,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="69">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -734,47 +755,50 @@
     <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="0"/>
     </xf>
+    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="top"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="top"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="top"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="top"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="top"/>
+    </xf>
     <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="top"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="top"/>
+      <alignment vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="top"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="top"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
@@ -1103,16 +1127,16 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="5.63"/>
     <col customWidth="1" min="2" max="2" width="39.13"/>
-    <col customWidth="1" min="3" max="3" width="9.38"/>
+    <col customWidth="1" min="3" max="3" width="14.25"/>
     <col customWidth="1" min="4" max="4" width="13.5"/>
-    <col customWidth="1" min="5" max="5" width="33.13"/>
-    <col customWidth="1" min="6" max="6" width="14.38"/>
-    <col customWidth="1" min="7" max="7" width="19.5"/>
+    <col customWidth="1" min="5" max="5" width="33.0"/>
+    <col customWidth="1" min="6" max="6" width="29.0"/>
+    <col customWidth="1" min="7" max="7" width="18.0"/>
     <col customWidth="1" min="8" max="8" width="15.63"/>
     <col customWidth="1" min="9" max="9" width="4.75"/>
-    <col customWidth="1" min="10" max="10" width="38.25"/>
+    <col customWidth="1" min="10" max="10" width="63.75"/>
     <col customWidth="1" min="11" max="11" width="56.13"/>
-    <col customWidth="1" min="12" max="12" width="8.5"/>
+    <col customWidth="1" min="12" max="12" width="12.0"/>
     <col customWidth="1" min="13" max="27" width="20.75"/>
   </cols>
   <sheetData>
@@ -3175,26 +3199,32 @@
         <v>65</v>
       </c>
       <c r="D65" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="E65" s="15" t="s">
         <v>113</v>
       </c>
-      <c r="E65" s="15" t="s">
+      <c r="F65" s="18" t="s">
+        <v>103</v>
+      </c>
+      <c r="G65" s="48" t="s">
+        <v>17</v>
+      </c>
+      <c r="H65" s="38">
+        <v>46083.0</v>
+      </c>
+      <c r="I65" s="31">
+        <v>1.0</v>
+      </c>
+      <c r="J65" s="31" t="s">
         <v>114</v>
       </c>
-      <c r="F65" s="18" t="s">
+      <c r="K65" s="31" t="s">
         <v>115</v>
       </c>
-      <c r="G65" s="18" t="s">
-        <v>116</v>
-      </c>
-      <c r="H65" s="38">
-        <v>45346.0</v>
-      </c>
-      <c r="I65" s="27">
-        <v>1.0</v>
-      </c>
-      <c r="J65" s="41"/>
-      <c r="K65" s="41"/>
-      <c r="L65" s="48"/>
+      <c r="L65" s="41" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="49"/>
@@ -3204,27 +3234,39 @@
       <c r="F66" s="52"/>
       <c r="G66" s="53"/>
       <c r="H66" s="50"/>
-      <c r="I66" s="30">
+      <c r="I66" s="32">
         <v>2.0</v>
       </c>
-      <c r="J66" s="45"/>
-      <c r="K66" s="45"/>
-      <c r="L66" s="54"/>
+      <c r="J66" s="32" t="s">
+        <v>116</v>
+      </c>
+      <c r="K66" s="32" t="s">
+        <v>117</v>
+      </c>
+      <c r="L66" s="45" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="67">
-      <c r="A67" s="55"/>
-      <c r="B67" s="56"/>
-      <c r="C67" s="57"/>
-      <c r="D67" s="58"/>
-      <c r="F67" s="58"/>
-      <c r="G67" s="59"/>
-      <c r="H67" s="56"/>
-      <c r="I67" s="27">
+      <c r="A67" s="54"/>
+      <c r="B67" s="55"/>
+      <c r="C67" s="56"/>
+      <c r="D67" s="57"/>
+      <c r="F67" s="57"/>
+      <c r="G67" s="58"/>
+      <c r="H67" s="55"/>
+      <c r="I67" s="31">
         <v>3.0</v>
       </c>
-      <c r="J67" s="41"/>
-      <c r="K67" s="41"/>
-      <c r="L67" s="48"/>
+      <c r="J67" s="31" t="s">
+        <v>118</v>
+      </c>
+      <c r="K67" s="31" t="s">
+        <v>119</v>
+      </c>
+      <c r="L67" s="41" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="49"/>
@@ -3234,27 +3276,28 @@
       <c r="F68" s="52"/>
       <c r="G68" s="53"/>
       <c r="H68" s="50"/>
-      <c r="I68" s="30">
+      <c r="I68" s="32">
         <v>4.0</v>
       </c>
-      <c r="J68" s="45"/>
-      <c r="K68" s="45"/>
-      <c r="L68" s="54"/>
+      <c r="J68" s="32" t="s">
+        <v>120</v>
+      </c>
+      <c r="K68" s="32" t="s">
+        <v>121</v>
+      </c>
+      <c r="L68" s="45" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="69">
-      <c r="A69" s="55"/>
-      <c r="B69" s="56"/>
-      <c r="C69" s="57"/>
-      <c r="D69" s="58"/>
-      <c r="F69" s="58"/>
-      <c r="G69" s="59"/>
-      <c r="H69" s="56"/>
-      <c r="I69" s="27">
-        <v>5.0</v>
-      </c>
-      <c r="J69" s="41"/>
-      <c r="K69" s="41"/>
-      <c r="L69" s="48"/>
+      <c r="A69" s="54"/>
+      <c r="B69" s="55"/>
+      <c r="C69" s="56"/>
+      <c r="D69" s="57"/>
+      <c r="F69" s="57"/>
+      <c r="G69" s="58"/>
+      <c r="H69" s="55"/>
+      <c r="L69" s="59"/>
     </row>
     <row r="70">
       <c r="A70" s="49"/>
@@ -3268,7 +3311,7 @@
       <c r="I70" s="30"/>
       <c r="J70" s="61"/>
       <c r="K70" s="61"/>
-      <c r="L70" s="54"/>
+      <c r="L70" s="62"/>
     </row>
   </sheetData>
   <mergeCells count="14">
@@ -3300,7 +3343,7 @@
     <dataValidation type="list" allowBlank="1" sqref="F2:F57 F59 F65">
       <formula1>"❌ NO PENDIENTE 🟡,✅ SÍ (Playwright) PASSED 🟢"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="L2:L64">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="L2:L68">
       <formula1>"Hecho,Pending"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3317,10 +3360,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="9" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2">
@@ -3350,145 +3393,145 @@
   </cols>
   <sheetData>
     <row r="45" ht="22.5" customHeight="1">
-      <c r="A45" s="62" t="s">
+      <c r="A45" s="63" t="s">
         <v>0</v>
       </c>
-      <c r="B45" s="63" t="s">
+      <c r="B45" s="64" t="s">
         <v>1</v>
       </c>
-      <c r="C45" s="63" t="s">
+      <c r="C45" s="64" t="s">
         <v>2</v>
       </c>
-      <c r="D45" s="63" t="s">
+      <c r="D45" s="64" t="s">
         <v>3</v>
       </c>
-      <c r="E45" s="63" t="s">
+      <c r="E45" s="64" t="s">
         <v>4</v>
       </c>
-      <c r="F45" s="63" t="s">
+      <c r="F45" s="64" t="s">
         <v>5</v>
       </c>
-      <c r="G45" s="63" t="s">
+      <c r="G45" s="64" t="s">
         <v>6</v>
       </c>
-      <c r="H45" s="63" t="s">
+      <c r="H45" s="64" t="s">
         <v>7</v>
       </c>
-      <c r="I45" s="62" t="s">
+      <c r="I45" s="63" t="s">
         <v>8</v>
       </c>
-      <c r="J45" s="63" t="s">
+      <c r="J45" s="64" t="s">
         <v>9</v>
       </c>
-      <c r="K45" s="63" t="s">
+      <c r="K45" s="64" t="s">
         <v>10</v>
       </c>
-      <c r="L45" s="63" t="s">
-        <v>119</v>
+      <c r="L45" s="64" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="46" ht="22.5" customHeight="1">
-      <c r="A46" s="64" t="s">
+      <c r="A46" s="65" t="s">
         <v>82</v>
       </c>
-      <c r="B46" s="65" t="s">
+      <c r="B46" s="66" t="s">
         <v>83</v>
       </c>
-      <c r="C46" s="65" t="s">
+      <c r="C46" s="66" t="s">
         <v>13</v>
       </c>
-      <c r="D46" s="65" t="s">
-        <v>113</v>
-      </c>
-      <c r="E46" s="65" t="s">
-        <v>120</v>
-      </c>
-      <c r="F46" s="65" t="s">
-        <v>117</v>
-      </c>
-      <c r="G46" s="65" t="s">
-        <v>116</v>
-      </c>
-      <c r="H46" s="66">
+      <c r="D46" s="66" t="s">
+        <v>125</v>
+      </c>
+      <c r="E46" s="66" t="s">
+        <v>126</v>
+      </c>
+      <c r="F46" s="66" t="s">
+        <v>122</v>
+      </c>
+      <c r="G46" s="66" t="s">
+        <v>127</v>
+      </c>
+      <c r="H46" s="67">
         <v>46066.0</v>
       </c>
-      <c r="I46" s="67">
+      <c r="I46" s="68">
         <v>1.0</v>
       </c>
-      <c r="J46" s="65" t="s">
-        <v>121</v>
-      </c>
-      <c r="K46" s="65" t="s">
-        <v>122</v>
-      </c>
-      <c r="L46" s="65" t="s">
-        <v>113</v>
+      <c r="J46" s="66" t="s">
+        <v>128</v>
+      </c>
+      <c r="K46" s="66" t="s">
+        <v>129</v>
+      </c>
+      <c r="L46" s="66" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="47" ht="22.5" customHeight="1">
-      <c r="A47" s="64"/>
-      <c r="B47" s="65"/>
-      <c r="C47" s="65"/>
-      <c r="D47" s="65"/>
-      <c r="E47" s="65"/>
-      <c r="F47" s="65"/>
-      <c r="G47" s="65"/>
-      <c r="H47" s="65"/>
-      <c r="I47" s="67">
+      <c r="A47" s="65"/>
+      <c r="B47" s="66"/>
+      <c r="C47" s="66"/>
+      <c r="D47" s="66"/>
+      <c r="E47" s="66"/>
+      <c r="F47" s="66"/>
+      <c r="G47" s="66"/>
+      <c r="H47" s="66"/>
+      <c r="I47" s="68">
         <v>2.0</v>
       </c>
-      <c r="J47" s="65" t="s">
+      <c r="J47" s="66" t="s">
         <v>85</v>
       </c>
-      <c r="K47" s="65" t="s">
+      <c r="K47" s="66" t="s">
         <v>86</v>
       </c>
-      <c r="L47" s="65" t="s">
-        <v>113</v>
+      <c r="L47" s="66" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="48" ht="22.5" customHeight="1">
-      <c r="A48" s="64"/>
-      <c r="B48" s="65"/>
-      <c r="C48" s="65"/>
-      <c r="D48" s="65"/>
-      <c r="E48" s="65"/>
-      <c r="F48" s="65"/>
-      <c r="G48" s="65"/>
-      <c r="H48" s="65"/>
-      <c r="I48" s="67">
+      <c r="A48" s="65"/>
+      <c r="B48" s="66"/>
+      <c r="C48" s="66"/>
+      <c r="D48" s="66"/>
+      <c r="E48" s="66"/>
+      <c r="F48" s="66"/>
+      <c r="G48" s="66"/>
+      <c r="H48" s="66"/>
+      <c r="I48" s="68">
         <v>3.0</v>
       </c>
-      <c r="J48" s="65" t="s">
+      <c r="J48" s="66" t="s">
         <v>87</v>
       </c>
-      <c r="K48" s="65" t="s">
+      <c r="K48" s="66" t="s">
         <v>88</v>
       </c>
-      <c r="L48" s="65" t="s">
-        <v>113</v>
+      <c r="L48" s="66" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="49" ht="22.5" customHeight="1">
-      <c r="A49" s="64"/>
-      <c r="B49" s="65"/>
-      <c r="C49" s="65"/>
-      <c r="D49" s="65"/>
-      <c r="E49" s="65"/>
-      <c r="F49" s="65"/>
-      <c r="G49" s="65"/>
-      <c r="H49" s="65"/>
-      <c r="I49" s="67">
+      <c r="A49" s="65"/>
+      <c r="B49" s="66"/>
+      <c r="C49" s="66"/>
+      <c r="D49" s="66"/>
+      <c r="E49" s="66"/>
+      <c r="F49" s="66"/>
+      <c r="G49" s="66"/>
+      <c r="H49" s="66"/>
+      <c r="I49" s="68">
         <v>4.0</v>
       </c>
-      <c r="J49" s="65" t="s">
+      <c r="J49" s="66" t="s">
         <v>89</v>
       </c>
-      <c r="K49" s="65" t="s">
+      <c r="K49" s="66" t="s">
         <v>90</v>
       </c>
-      <c r="L49" s="65" t="s">
-        <v>113</v>
+      <c r="L49" s="66" t="s">
+        <v>125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Actualizar el archivo QA_Roadmap_Natalia.xlsx con nuevos datos
</commit_message>
<xml_diff>
--- a/docs/QA_Roadmap_Natalia.xlsx
+++ b/docs/QA_Roadmap_Natalia.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="162">
   <si>
     <t>ID</t>
   </si>
@@ -525,6 +525,102 @@
     <t>El producto NO se eliminó y el badge sigue en "1".</t>
   </si>
   <si>
+    <t>TC-15</t>
+  </si>
+  <si>
+    <t>Validar proceso de compra completo con checkout.</t>
+  </si>
+  <si>
+    <t>TC-16</t>
+  </si>
+  <si>
+    <t>Validar respuesta GET de lista de usuarios (API)</t>
+  </si>
+  <si>
+    <t>P1 (Alta)</t>
+  </si>
+  <si>
+    <t>N/A (API Request)</t>
+  </si>
+  <si>
+    <t>Enviar petición GET al endpoint de usuarios.</t>
+  </si>
+  <si>
+    <t>El servidor procesa la solicitud.</t>
+  </si>
+  <si>
+    <t>Validar Status Code.</t>
+  </si>
+  <si>
+    <t>El Status Code es 200 (OK).</t>
+  </si>
+  <si>
+    <t>Validar payload de respuesta (JSON).</t>
+  </si>
+  <si>
+    <t>El JSON contiene una lista de usuarios (data.length &gt; 0).</t>
+  </si>
+  <si>
+    <t>TC-17</t>
+  </si>
+  <si>
+    <t>Validar creación de usuario mediante POST (API)</t>
+  </si>
+  <si>
+    <t>Enviar petición POST con payload JSON (nombre y trabajo).</t>
+  </si>
+  <si>
+    <t>El servidor recibe los datos para creación.</t>
+  </si>
+  <si>
+    <t>El Status Code es 201 (Created).</t>
+  </si>
+  <si>
+    <t>Validar confirmación de creación.</t>
+  </si>
+  <si>
+    <t>El JSON de respuesta contiene el 'id' generado y los datos enviados.</t>
+  </si>
+  <si>
+    <t>TC-18</t>
+  </si>
+  <si>
+    <t>Validar actualización de usuario mediante PUT (API)</t>
+  </si>
+  <si>
+    <t>Por Automatizar</t>
+  </si>
+  <si>
+    <t>Enviar petición PUT a /users/1 con nuevo rol.</t>
+  </si>
+  <si>
+    <t>El servidor procesa la solicitud de actualización.</t>
+  </si>
+  <si>
+    <t>Validar JSON de respuesta.</t>
+  </si>
+  <si>
+    <t>El JSON refleja el cambio enviado (ej. "Lead QA").</t>
+  </si>
+  <si>
+    <t>TC-19</t>
+  </si>
+  <si>
+    <t>Validar eliminación de usuario mediante DELETE (API)</t>
+  </si>
+  <si>
+    <t>Enviar petición DELETE al endpoint /users/1.</t>
+  </si>
+  <si>
+    <t>El servidor procesa la orden de borrado.</t>
+  </si>
+  <si>
+    <t>Validar Status Code de eliminación.</t>
+  </si>
+  <si>
+    <t>El Status Code es 200 (OK) o 204 (No Content).</t>
+  </si>
+  <si>
     <t>❌ NO</t>
   </si>
   <si>
@@ -553,11 +649,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="165" formatCode="d/MM/yyyy"/>
+    <numFmt numFmtId="166" formatCode="dd-mm-yyyy"/>
+    <numFmt numFmtId="167" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -578,6 +676,15 @@
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <color rgb="FF1F1F1F"/>
+      <name val="&quot;Google Sans Text&quot;"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF1F1F1F"/>
+      <name val="&quot;Google Sans Text&quot;"/>
     </font>
   </fonts>
   <fills count="5">
@@ -612,7 +719,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="77">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -799,6 +906,28 @@
     </xf>
     <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="1" numFmtId="166" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="top"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="167" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
@@ -827,16 +956,6 @@
       <font/>
       <fill>
         <patternFill patternType="none"/>
-      </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF535FC1"/>
-          <bgColor rgb="FF535FC1"/>
-        </patternFill>
       </fill>
       <border/>
     </dxf>
@@ -861,6 +980,16 @@
       <border/>
     </dxf>
     <dxf>
+      <font/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF535FC1"/>
+          <bgColor rgb="FF535FC1"/>
+        </patternFill>
+      </fill>
+      <border/>
+    </dxf>
+    <dxf>
       <border>
         <left style="thin">
           <color rgb="FF535FC1"/>
@@ -877,11 +1006,27 @@
       </border>
     </dxf>
   </dxfs>
-  <tableStyles count="1">
+  <tableStyles count="5">
+    <tableStyle count="2" pivot="0" name="Actualización de Test Case Auto-style">
+      <tableStyleElement dxfId="1" type="firstRowStripe"/>
+      <tableStyleElement dxfId="2" type="secondRowStripe"/>
+    </tableStyle>
+    <tableStyle count="2" pivot="0" name="Actualización de Test Case Auto-style 2">
+      <tableStyleElement dxfId="1" type="firstRowStripe"/>
+      <tableStyleElement dxfId="2" type="secondRowStripe"/>
+    </tableStyle>
+    <tableStyle count="2" pivot="0" name="Actualización de Test Case Auto-style 3">
+      <tableStyleElement dxfId="1" type="firstRowStripe"/>
+      <tableStyleElement dxfId="2" type="secondRowStripe"/>
+    </tableStyle>
+    <tableStyle count="2" pivot="0" name="Actualización de Test Case Auto-style 4">
+      <tableStyleElement dxfId="1" type="firstRowStripe"/>
+      <tableStyleElement dxfId="2" type="secondRowStripe"/>
+    </tableStyle>
     <tableStyle count="4" pivot="0" name="Hoja 2-style">
-      <tableStyleElement dxfId="1" type="headerRow"/>
-      <tableStyleElement dxfId="2" type="firstRowStripe"/>
-      <tableStyleElement dxfId="3" type="secondRowStripe"/>
+      <tableStyleElement dxfId="3" type="headerRow"/>
+      <tableStyleElement dxfId="1" type="firstRowStripe"/>
+      <tableStyleElement dxfId="2" type="secondRowStripe"/>
       <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
     </tableStyle>
   </tableStyles>
@@ -905,7 +1050,47 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A45:L49" displayName="Tabla_1" name="Tabla_1" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="F76:G76" displayName="Table_1" name="Table_1" id="1">
+  <tableColumns count="2">
+    <tableColumn name="Column1" id="1"/>
+    <tableColumn name="Column2" id="2"/>
+  </tableColumns>
+  <tableStyleInfo name="Actualización de Test Case Auto-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="F79:G79" displayName="Table_2" name="Table_2" id="2">
+  <tableColumns count="2">
+    <tableColumn name="Column1" id="1"/>
+    <tableColumn name="Column2" id="2"/>
+  </tableColumns>
+  <tableStyleInfo name="Actualización de Test Case Auto-style 2" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="F83:G83" displayName="Table_3" name="Table_3" id="3">
+  <tableColumns count="2">
+    <tableColumn name="Column1" id="1"/>
+    <tableColumn name="Column2" id="2"/>
+  </tableColumns>
+  <tableStyleInfo name="Actualización de Test Case Auto-style 3" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="F86:G86" displayName="Table_4" name="Table_4" id="4">
+  <tableColumns count="2">
+    <tableColumn name="Column1" id="1"/>
+    <tableColumn name="Column2" id="2"/>
+  </tableColumns>
+  <tableStyleInfo name="Actualización de Test Case Auto-style 4" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A45:L49" displayName="Tabla_1" name="Tabla_1" id="5">
   <tableColumns count="12">
     <tableColumn name="ID" id="1"/>
     <tableColumn name="Título del Test" id="2"/>
@@ -1126,7 +1311,7 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="5.63"/>
-    <col customWidth="1" min="2" max="2" width="39.13"/>
+    <col customWidth="1" min="2" max="2" width="46.5"/>
     <col customWidth="1" min="3" max="3" width="14.25"/>
     <col customWidth="1" min="4" max="4" width="13.5"/>
     <col customWidth="1" min="5" max="5" width="33.0"/>
@@ -3313,6 +3498,402 @@
       <c r="K70" s="61"/>
       <c r="L70" s="62"/>
     </row>
+    <row r="71">
+      <c r="A71" s="27" t="s">
+        <v>122</v>
+      </c>
+      <c r="B71" s="37" t="s">
+        <v>123</v>
+      </c>
+      <c r="C71" s="46" t="s">
+        <v>13</v>
+      </c>
+      <c r="D71" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="E71" s="63"/>
+      <c r="F71" s="18" t="s">
+        <v>103</v>
+      </c>
+      <c r="G71" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="H71" s="64">
+        <v>46085.0</v>
+      </c>
+      <c r="I71" s="31">
+        <v>1.0</v>
+      </c>
+      <c r="J71" s="31" t="s">
+        <v>114</v>
+      </c>
+      <c r="K71" s="31" t="s">
+        <v>115</v>
+      </c>
+      <c r="L71" s="41" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="49"/>
+      <c r="B72" s="50"/>
+      <c r="C72" s="51"/>
+      <c r="D72" s="52"/>
+      <c r="E72" s="60"/>
+      <c r="F72" s="52"/>
+      <c r="G72" s="52"/>
+      <c r="H72" s="50"/>
+      <c r="I72" s="32">
+        <v>2.0</v>
+      </c>
+      <c r="J72" s="32" t="s">
+        <v>116</v>
+      </c>
+      <c r="K72" s="32" t="s">
+        <v>117</v>
+      </c>
+      <c r="L72" s="45" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="54"/>
+      <c r="B73" s="55"/>
+      <c r="C73" s="56"/>
+      <c r="D73" s="57"/>
+      <c r="E73" s="63"/>
+      <c r="F73" s="57"/>
+      <c r="G73" s="57"/>
+      <c r="H73" s="55"/>
+      <c r="I73" s="31">
+        <v>3.0</v>
+      </c>
+      <c r="L73" s="41" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="49"/>
+      <c r="B74" s="50"/>
+      <c r="C74" s="51"/>
+      <c r="D74" s="52"/>
+      <c r="E74" s="60"/>
+      <c r="F74" s="52"/>
+      <c r="G74" s="52"/>
+      <c r="H74" s="50"/>
+      <c r="I74" s="32">
+        <v>4.0</v>
+      </c>
+      <c r="L74" s="45" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="65" t="s">
+        <v>124</v>
+      </c>
+      <c r="B76" s="65" t="s">
+        <v>125</v>
+      </c>
+      <c r="C76" s="65" t="s">
+        <v>126</v>
+      </c>
+      <c r="D76" s="66" t="s">
+        <v>14</v>
+      </c>
+      <c r="E76" s="65" t="s">
+        <v>127</v>
+      </c>
+      <c r="F76" s="66" t="s">
+        <v>103</v>
+      </c>
+      <c r="G76" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="H76" s="67">
+        <v>46105.0</v>
+      </c>
+      <c r="I76" s="65">
+        <v>1.0</v>
+      </c>
+      <c r="J76" s="65" t="s">
+        <v>128</v>
+      </c>
+      <c r="K76" s="65" t="s">
+        <v>129</v>
+      </c>
+      <c r="L76" s="68" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="69"/>
+      <c r="B77" s="69"/>
+      <c r="C77" s="69"/>
+      <c r="D77" s="69"/>
+      <c r="E77" s="69"/>
+      <c r="F77" s="69"/>
+      <c r="G77" s="69"/>
+      <c r="H77" s="69"/>
+      <c r="I77" s="65">
+        <v>2.0</v>
+      </c>
+      <c r="J77" s="65" t="s">
+        <v>130</v>
+      </c>
+      <c r="K77" s="65" t="s">
+        <v>131</v>
+      </c>
+      <c r="L77" s="68" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="69"/>
+      <c r="B78" s="69"/>
+      <c r="C78" s="69"/>
+      <c r="D78" s="69"/>
+      <c r="E78" s="69"/>
+      <c r="F78" s="69"/>
+      <c r="G78" s="69"/>
+      <c r="H78" s="69"/>
+      <c r="I78" s="65">
+        <v>3.0</v>
+      </c>
+      <c r="J78" s="65" t="s">
+        <v>132</v>
+      </c>
+      <c r="K78" s="65" t="s">
+        <v>133</v>
+      </c>
+      <c r="L78" s="68" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="65" t="s">
+        <v>134</v>
+      </c>
+      <c r="B79" s="65" t="s">
+        <v>135</v>
+      </c>
+      <c r="C79" s="65" t="s">
+        <v>13</v>
+      </c>
+      <c r="D79" s="66" t="s">
+        <v>14</v>
+      </c>
+      <c r="E79" s="65" t="s">
+        <v>127</v>
+      </c>
+      <c r="F79" s="66" t="s">
+        <v>103</v>
+      </c>
+      <c r="G79" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="H79" s="67">
+        <v>46105.0</v>
+      </c>
+      <c r="I79" s="65">
+        <v>1.0</v>
+      </c>
+      <c r="J79" s="65" t="s">
+        <v>136</v>
+      </c>
+      <c r="K79" s="65" t="s">
+        <v>137</v>
+      </c>
+      <c r="L79" s="68" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="69"/>
+      <c r="B80" s="69"/>
+      <c r="C80" s="69"/>
+      <c r="D80" s="69"/>
+      <c r="E80" s="69"/>
+      <c r="F80" s="69"/>
+      <c r="G80" s="69"/>
+      <c r="H80" s="69"/>
+      <c r="I80" s="65">
+        <v>2.0</v>
+      </c>
+      <c r="J80" s="65" t="s">
+        <v>130</v>
+      </c>
+      <c r="K80" s="65" t="s">
+        <v>138</v>
+      </c>
+      <c r="L80" s="68" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="69"/>
+      <c r="B81" s="69"/>
+      <c r="C81" s="69"/>
+      <c r="D81" s="69"/>
+      <c r="E81" s="69"/>
+      <c r="F81" s="69"/>
+      <c r="G81" s="69"/>
+      <c r="H81" s="69"/>
+      <c r="I81" s="65">
+        <v>3.0</v>
+      </c>
+      <c r="J81" s="65" t="s">
+        <v>139</v>
+      </c>
+      <c r="K81" s="65" t="s">
+        <v>140</v>
+      </c>
+      <c r="L81" s="68" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="70" t="s">
+        <v>141</v>
+      </c>
+      <c r="B83" s="65" t="s">
+        <v>142</v>
+      </c>
+      <c r="C83" s="65" t="s">
+        <v>126</v>
+      </c>
+      <c r="D83" s="65" t="s">
+        <v>143</v>
+      </c>
+      <c r="E83" s="65" t="s">
+        <v>127</v>
+      </c>
+      <c r="F83" s="66" t="s">
+        <v>103</v>
+      </c>
+      <c r="G83" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="H83" s="67">
+        <v>46107.0</v>
+      </c>
+      <c r="I83" s="65">
+        <v>1.0</v>
+      </c>
+      <c r="J83" s="65" t="s">
+        <v>144</v>
+      </c>
+      <c r="K83" s="65" t="s">
+        <v>145</v>
+      </c>
+      <c r="L83" s="68" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="69"/>
+      <c r="B84" s="69"/>
+      <c r="C84" s="69"/>
+      <c r="D84" s="69"/>
+      <c r="E84" s="69"/>
+      <c r="F84" s="69"/>
+      <c r="G84" s="69"/>
+      <c r="H84" s="69"/>
+      <c r="I84" s="65">
+        <v>2.0</v>
+      </c>
+      <c r="J84" s="65" t="s">
+        <v>130</v>
+      </c>
+      <c r="K84" s="65" t="s">
+        <v>131</v>
+      </c>
+      <c r="L84" s="68" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="69"/>
+      <c r="B85" s="69"/>
+      <c r="C85" s="69"/>
+      <c r="D85" s="69"/>
+      <c r="E85" s="69"/>
+      <c r="F85" s="69"/>
+      <c r="G85" s="69"/>
+      <c r="H85" s="69"/>
+      <c r="I85" s="65">
+        <v>3.0</v>
+      </c>
+      <c r="J85" s="65" t="s">
+        <v>146</v>
+      </c>
+      <c r="K85" s="65" t="s">
+        <v>147</v>
+      </c>
+      <c r="L85" s="68" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="70" t="s">
+        <v>148</v>
+      </c>
+      <c r="B86" s="65" t="s">
+        <v>149</v>
+      </c>
+      <c r="C86" s="65" t="s">
+        <v>126</v>
+      </c>
+      <c r="D86" s="65" t="s">
+        <v>143</v>
+      </c>
+      <c r="E86" s="65" t="s">
+        <v>127</v>
+      </c>
+      <c r="F86" s="66" t="s">
+        <v>103</v>
+      </c>
+      <c r="G86" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="H86" s="67">
+        <v>46107.0</v>
+      </c>
+      <c r="I86" s="65">
+        <v>1.0</v>
+      </c>
+      <c r="J86" s="65" t="s">
+        <v>150</v>
+      </c>
+      <c r="K86" s="65" t="s">
+        <v>151</v>
+      </c>
+      <c r="L86" s="68" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="69"/>
+      <c r="B87" s="69"/>
+      <c r="C87" s="69"/>
+      <c r="D87" s="69"/>
+      <c r="E87" s="69"/>
+      <c r="F87" s="69"/>
+      <c r="G87" s="69"/>
+      <c r="H87" s="69"/>
+      <c r="I87" s="65">
+        <v>2.0</v>
+      </c>
+      <c r="J87" s="65" t="s">
+        <v>152</v>
+      </c>
+      <c r="K87" s="65" t="s">
+        <v>153</v>
+      </c>
+      <c r="L87" s="68" t="s">
+        <v>20</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="14">
     <mergeCell ref="E31:E34"/>
@@ -3331,23 +3912,29 @@
     <mergeCell ref="E27:E30"/>
   </mergeCells>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:C59 C65">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:C59 C65 C71">
       <formula1>"P0 (Crítica),P0"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="D2:D57 D59 D65">
+    <dataValidation type="list" allowBlank="1" sqref="D2:D57 D59 D65 D71 D76 D79">
       <formula1>"Finalizado,Pendiente"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="G2:G57 G59 G65">
+    <dataValidation type="list" allowBlank="1" sqref="G2:G57 G59 G65 G71 G76 G79 G83 G86">
       <formula1>"PENDIENTE 🟡,PASSED 🟢"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="F2:F57 F59 F65">
+    <dataValidation type="list" allowBlank="1" sqref="F2:F57 F59 F65 F71 F76 F79 F83 F86">
       <formula1>"❌ NO PENDIENTE 🟡,✅ SÍ (Playwright) PASSED 🟢"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="L2:L68">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="L2:L68 L71:L74 L76:L81 L83:L87">
       <formula1>"Hecho,Pending"</formula1>
     </dataValidation>
   </dataValidations>
   <drawing r:id="rId1"/>
+  <tableParts count="4">
+    <tablePart r:id="rId6"/>
+    <tablePart r:id="rId7"/>
+    <tablePart r:id="rId8"/>
+    <tablePart r:id="rId9"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -3360,10 +3947,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="9" t="s">
-        <v>122</v>
+        <v>154</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>123</v>
+        <v>155</v>
       </c>
     </row>
     <row r="2">
@@ -3393,145 +3980,145 @@
   </cols>
   <sheetData>
     <row r="45" ht="22.5" customHeight="1">
-      <c r="A45" s="63" t="s">
+      <c r="A45" s="71" t="s">
         <v>0</v>
       </c>
-      <c r="B45" s="64" t="s">
+      <c r="B45" s="72" t="s">
         <v>1</v>
       </c>
-      <c r="C45" s="64" t="s">
+      <c r="C45" s="72" t="s">
         <v>2</v>
       </c>
-      <c r="D45" s="64" t="s">
+      <c r="D45" s="72" t="s">
         <v>3</v>
       </c>
-      <c r="E45" s="64" t="s">
+      <c r="E45" s="72" t="s">
         <v>4</v>
       </c>
-      <c r="F45" s="64" t="s">
+      <c r="F45" s="72" t="s">
         <v>5</v>
       </c>
-      <c r="G45" s="64" t="s">
+      <c r="G45" s="72" t="s">
         <v>6</v>
       </c>
-      <c r="H45" s="64" t="s">
+      <c r="H45" s="72" t="s">
         <v>7</v>
       </c>
-      <c r="I45" s="63" t="s">
+      <c r="I45" s="71" t="s">
         <v>8</v>
       </c>
-      <c r="J45" s="64" t="s">
+      <c r="J45" s="72" t="s">
         <v>9</v>
       </c>
-      <c r="K45" s="64" t="s">
+      <c r="K45" s="72" t="s">
         <v>10</v>
       </c>
-      <c r="L45" s="64" t="s">
-        <v>124</v>
+      <c r="L45" s="72" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="46" ht="22.5" customHeight="1">
-      <c r="A46" s="65" t="s">
+      <c r="A46" s="73" t="s">
         <v>82</v>
       </c>
-      <c r="B46" s="66" t="s">
+      <c r="B46" s="74" t="s">
         <v>83</v>
       </c>
-      <c r="C46" s="66" t="s">
+      <c r="C46" s="74" t="s">
         <v>13</v>
       </c>
-      <c r="D46" s="66" t="s">
-        <v>125</v>
-      </c>
-      <c r="E46" s="66" t="s">
-        <v>126</v>
-      </c>
-      <c r="F46" s="66" t="s">
-        <v>122</v>
-      </c>
-      <c r="G46" s="66" t="s">
-        <v>127</v>
-      </c>
-      <c r="H46" s="67">
+      <c r="D46" s="74" t="s">
+        <v>157</v>
+      </c>
+      <c r="E46" s="74" t="s">
+        <v>158</v>
+      </c>
+      <c r="F46" s="74" t="s">
+        <v>154</v>
+      </c>
+      <c r="G46" s="74" t="s">
+        <v>159</v>
+      </c>
+      <c r="H46" s="75">
         <v>46066.0</v>
       </c>
-      <c r="I46" s="68">
+      <c r="I46" s="76">
         <v>1.0</v>
       </c>
-      <c r="J46" s="66" t="s">
-        <v>128</v>
-      </c>
-      <c r="K46" s="66" t="s">
-        <v>129</v>
-      </c>
-      <c r="L46" s="66" t="s">
-        <v>125</v>
+      <c r="J46" s="74" t="s">
+        <v>160</v>
+      </c>
+      <c r="K46" s="74" t="s">
+        <v>161</v>
+      </c>
+      <c r="L46" s="74" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="47" ht="22.5" customHeight="1">
-      <c r="A47" s="65"/>
-      <c r="B47" s="66"/>
-      <c r="C47" s="66"/>
-      <c r="D47" s="66"/>
-      <c r="E47" s="66"/>
-      <c r="F47" s="66"/>
-      <c r="G47" s="66"/>
-      <c r="H47" s="66"/>
-      <c r="I47" s="68">
+      <c r="A47" s="73"/>
+      <c r="B47" s="74"/>
+      <c r="C47" s="74"/>
+      <c r="D47" s="74"/>
+      <c r="E47" s="74"/>
+      <c r="F47" s="74"/>
+      <c r="G47" s="74"/>
+      <c r="H47" s="74"/>
+      <c r="I47" s="76">
         <v>2.0</v>
       </c>
-      <c r="J47" s="66" t="s">
+      <c r="J47" s="74" t="s">
         <v>85</v>
       </c>
-      <c r="K47" s="66" t="s">
+      <c r="K47" s="74" t="s">
         <v>86</v>
       </c>
-      <c r="L47" s="66" t="s">
-        <v>125</v>
+      <c r="L47" s="74" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="48" ht="22.5" customHeight="1">
-      <c r="A48" s="65"/>
-      <c r="B48" s="66"/>
-      <c r="C48" s="66"/>
-      <c r="D48" s="66"/>
-      <c r="E48" s="66"/>
-      <c r="F48" s="66"/>
-      <c r="G48" s="66"/>
-      <c r="H48" s="66"/>
-      <c r="I48" s="68">
+      <c r="A48" s="73"/>
+      <c r="B48" s="74"/>
+      <c r="C48" s="74"/>
+      <c r="D48" s="74"/>
+      <c r="E48" s="74"/>
+      <c r="F48" s="74"/>
+      <c r="G48" s="74"/>
+      <c r="H48" s="74"/>
+      <c r="I48" s="76">
         <v>3.0</v>
       </c>
-      <c r="J48" s="66" t="s">
+      <c r="J48" s="74" t="s">
         <v>87</v>
       </c>
-      <c r="K48" s="66" t="s">
+      <c r="K48" s="74" t="s">
         <v>88</v>
       </c>
-      <c r="L48" s="66" t="s">
-        <v>125</v>
+      <c r="L48" s="74" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="49" ht="22.5" customHeight="1">
-      <c r="A49" s="65"/>
-      <c r="B49" s="66"/>
-      <c r="C49" s="66"/>
-      <c r="D49" s="66"/>
-      <c r="E49" s="66"/>
-      <c r="F49" s="66"/>
-      <c r="G49" s="66"/>
-      <c r="H49" s="66"/>
-      <c r="I49" s="68">
+      <c r="A49" s="73"/>
+      <c r="B49" s="74"/>
+      <c r="C49" s="74"/>
+      <c r="D49" s="74"/>
+      <c r="E49" s="74"/>
+      <c r="F49" s="74"/>
+      <c r="G49" s="74"/>
+      <c r="H49" s="74"/>
+      <c r="I49" s="76">
         <v>4.0</v>
       </c>
-      <c r="J49" s="66" t="s">
+      <c r="J49" s="74" t="s">
         <v>89</v>
       </c>
-      <c r="K49" s="66" t="s">
+      <c r="K49" s="74" t="s">
         <v>90</v>
       </c>
-      <c r="L49" s="66" t="s">
-        <v>125</v>
+      <c r="L49" s="74" t="s">
+        <v>157</v>
       </c>
     </row>
   </sheetData>

</xml_diff>